<commit_message>
feat: shopper money flow + Master admin Withdrawals
Shopper website:
- Reserve Offer shows claim-slot use; separate Confirm Reservation screen (exact deadline, slot N of 5)
- Wallet: pending approval total, Wallet Activity with filters, Reward Details timeline
- 5-step withdrawal: any amount, locked method + request a change, SMS, confirm checkbox,
  Requested/Processing/Paid tracker, Additional review needed pop-up
- New GET /wallet/activity/

Admin Withdrawals (Master Sheet 1):
- Safe requests go straight to Ready for Batch; review-rule matches go to Manual Review
- Tabs Ready for Batch / Manual Review / Processing / Completed / Failed with batch summary
- Create batch downloads the PayPal Payouts CSV; import PayPal results (match on Withdrawal ID,
  partial success, idempotent); Failed retryable (retry) or permanent (returned to balance)
- Rejection requires a customer-facing reason; every decision audit-logged
- Needs Attention counts failed payouts

Tracker: 99 of 150 completed
</commit_message>
<xml_diff>
--- a/docs/client-requirements/Nibbl_Master_Requirements_Tracker.xlsx
+++ b/docs/client-requirements/Nibbl_Master_Requirements_Tracker.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1550" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1545" uniqueCount="704">
   <si>
     <t xml:space="preserve">Nibbl AI — Master Requirements Tracker</t>
   </si>
@@ -770,13 +770,13 @@
     <t xml:space="preserve">Confirm Reservation screen: slot X of 5, exact deadline, Confirm &amp; Reserve (slot consumed only here)</t>
   </si>
   <si>
-    <t xml:space="preserve">Claim reserves directly after the consent step.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claim an offer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Separate confirmation screen showing slot use + exact deadline before reserving not built on the website.</t>
+    <t xml:space="preserve">Slot use shown on Reserve Offer; separate Confirm screen with product, retailer, reward, exact deadline and resulting slot use.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → offer → Continue → Confirm &amp; Reserve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claim an offer; check the deadline is 7 days out.</t>
   </si>
   <si>
     <t xml:space="preserve">#18</t>
@@ -1553,19 +1553,22 @@
     <t xml:space="preserve">Wallet activity with filters (rebates, reviews, referrals, withdrawals) + statuses</t>
   </si>
   <si>
-    <t xml:space="preserve">Activity list.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open activity.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filter tabs not built.</t>
+    <t xml:space="preserve">New /wallet/activity/: All / Rebates / Reviews / Referrals / Withdrawals tabs, grouped Pending / In progress / Available / Completed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → Wallet → Wallet Activity</t>
   </si>
   <si>
     <t xml:space="preserve">Reward details (timeline: submitted → under review → available)</t>
   </si>
   <si>
-    <t xml:space="preserve">Not built on the website.</t>
+    <t xml:space="preserve">Reward Details pop-up with timeline, reward type, campaign, receipt date, reference.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → Wallet → tap an item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open a pending rebate.</t>
   </si>
   <si>
     <t xml:space="preserve">Payout methods: one PayPal/Venmo identity per account; locked; change via request</t>
@@ -1583,7 +1586,7 @@
     <t xml:space="preserve">Amount → locked method → SMS code → confirm (checkbox) → requested status tracker</t>
   </si>
   <si>
-    <t xml:space="preserve">Amount, method, SMS code, submit.</t>
+    <t xml:space="preserve">All five steps incl. any amount, locked method + Request a change, SMS, confirm checkbox, Requested / Processing / Paid tracker.</t>
   </si>
   <si>
     <t xml:space="preserve">Website → Wallet → Withdraw</t>
@@ -1592,31 +1595,34 @@
     <t xml:space="preserve">Withdraw a small amount.</t>
   </si>
   <si>
-    <t xml:space="preserve">Twilio approved — retest SMS. Confirm-step checkbox and Requested/Processing/Paid tracker not built.</t>
+    <t xml:space="preserve">Twilio approved — retest the SMS step on production, then Completed.</t>
   </si>
   <si>
     <t xml:space="preserve">'Additional review needed' popup; status stays Processing</t>
   </si>
   <si>
-    <t xml:space="preserve">Review routing in Admin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trigger a review rule.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shopper popup not built.</t>
+    <t xml:space="preserve">Pop-up with Got it; request shows Processing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → Wallet → Withdraw over the review threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Withdraw above $25.</t>
   </si>
   <si>
     <t xml:space="preserve">Withdrawal failed / rejected balance handling</t>
   </si>
   <si>
-    <t xml:space="preserve">Rejected returns the amount (hold released).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reject a withdrawal.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Failed (retryable vs permanent) handling waits on PayPal results import.</t>
+    <t xml:space="preserve">Rejected: full amount back to the balance with the reason. Failed (from PayPal results): retryable stays reserved (Retry), permanent returns the amount (Return to balance).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopper Website + Admin Dashboard + Backend / API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → Wallet Activity; Admin → Withdrawals → Failed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Import a FAILED result, then Return to balance.</t>
   </si>
   <si>
     <t xml:space="preserve">#43</t>
@@ -1715,7 +1721,7 @@
     <t xml:space="preserve">Change date range.</t>
   </si>
   <si>
-    <t xml:space="preserve">Brand category filter (brands have no category); failed payouts wait on results import.</t>
+    <t xml:space="preserve">Brand category filter (brands have no category). Failed payouts count is now live.</t>
   </si>
   <si>
     <t xml:space="preserve">#42</t>
@@ -1727,37 +1733,55 @@
     <t xml:space="preserve">Tabs: Ready for Batch, Manual Review, Processing, Completed, Failed; batch summary (PayPal fees)</t>
   </si>
   <si>
-    <t xml:space="preserve">Batches, approve/reject, manual review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Admin → Withdraw Request / Payout Reviews</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create a batch.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tab set and batch-cost summary per mockup; no Failed tab.</t>
+    <t xml:space="preserve">All five tabs with counts; safe requests enter Ready for Batch automatically; live batch summary (count, payouts, est. PayPal fees, total).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin → Withdrawals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Select requests; watch the summary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PayPal fee estimate = $0.25 per payout (configurable on the server).</t>
   </si>
   <si>
     <t xml:space="preserve">Create batch, download PayPal file</t>
   </si>
   <si>
-    <t xml:space="preserve">Admin → Withdraw Request</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Download a batch file.</t>
+    <t xml:space="preserve">Create Batch from selected requests downloads the PayPal Payouts CSV (Reference ID = Withdrawal ID); past batches can be downloaded again; an exported request can't join a second batch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin → Withdrawals → Create Batch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a batch; upload the file to PayPal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check the file against PayPal's current Payouts template on first use.</t>
   </si>
   <si>
     <t xml:space="preserve">Import PayPal results (Paid / Failed, partial success, idempotent, match by Withdrawal ID)</t>
   </si>
   <si>
+    <t xml:space="preserve">Import PayPal Results: matches Reference ID; SUCCESS → Paid, failures → Failed (retryable or permanent); partial success; re-import changes nothing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin → Withdrawals → Import PayPal Results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Import a results CSV twice.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Manual review: flag reason + history; approve / reject with customer-facing reason; audit</t>
   </si>
   <si>
-    <t xml:space="preserve">Admin → Payout Reviews</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approve a flagged request.</t>
+    <t xml:space="preserve">Manual Review panel: flag reason, shopper history, Approve (→ Ready for Batch) / Reject with required reason; every decision audit-logged.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin → Withdrawals → Manual Review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approve and reject a flagged request.</t>
   </si>
   <si>
     <t xml:space="preserve">#43, #51</t>
@@ -2973,11 +2997,11 @@
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"Completed")</f>
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"In Progress")</f>
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"In Review")</f>
@@ -2985,11 +3009,11 @@
       </c>
       <c r="G5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"Planned")</f>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H5" s="5" t="n">
         <f aca="false">IF(C5&gt;0,D5/C5,0)</f>
-        <v>0.613333333333333</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4733,7 +4757,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="9" t="n">
         <v>50</v>
       </c>
@@ -4747,23 +4771,21 @@
         <v>247</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>236</v>
+        <v>207</v>
       </c>
       <c r="H58" s="10" t="s">
         <v>208</v>
       </c>
       <c r="I58" s="10" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="J58" s="10" t="s">
-        <v>248</v>
-      </c>
-      <c r="K58" s="10" t="s">
         <v>249</v>
       </c>
+      <c r="K58" s="10"/>
       <c r="L58" s="12"/>
       <c r="M58" s="13" t="s">
         <v>250</v>
@@ -7103,7 +7125,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B126" s="9" t="n">
         <v>118</v>
       </c>
@@ -7117,23 +7139,21 @@
         <v>508</v>
       </c>
       <c r="F126" s="11" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G126" s="10" t="s">
-        <v>236</v>
+        <v>207</v>
       </c>
       <c r="H126" s="10" t="s">
         <v>208</v>
       </c>
       <c r="I126" s="10" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="J126" s="10" t="s">
-        <v>509</v>
-      </c>
-      <c r="K126" s="10" t="s">
-        <v>510</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="K126" s="10"/>
       <c r="L126" s="12"/>
       <c r="M126" s="13" t="s">
         <v>506</v>
@@ -7147,29 +7167,27 @@
         <v>503</v>
       </c>
       <c r="D127" s="10" t="s">
+        <v>510</v>
+      </c>
+      <c r="E127" s="10" t="s">
         <v>511</v>
       </c>
-      <c r="E127" s="10" t="s">
-        <v>31</v>
-      </c>
       <c r="F127" s="11" t="s">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="G127" s="10" t="s">
-        <v>236</v>
+        <v>207</v>
       </c>
       <c r="H127" s="10" t="s">
         <v>208</v>
       </c>
       <c r="I127" s="10" t="s">
-        <v>31</v>
+        <v>512</v>
       </c>
       <c r="J127" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="K127" s="10" t="s">
-        <v>512</v>
-      </c>
+        <v>513</v>
+      </c>
+      <c r="K127" s="10"/>
       <c r="L127" s="12"/>
       <c r="M127" s="13" t="s">
         <v>506</v>
@@ -7183,7 +7201,7 @@
         <v>503</v>
       </c>
       <c r="D128" s="10" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="E128" s="10" t="s">
         <v>59</v>
@@ -7201,26 +7219,26 @@
         <v>505</v>
       </c>
       <c r="J128" s="10" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="K128" s="10"/>
       <c r="L128" s="12"/>
       <c r="M128" s="13" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="129" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B129" s="9" t="n">
         <v>121</v>
       </c>
       <c r="C129" s="10" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D129" s="10" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E129" s="10" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F129" s="11" t="s">
         <v>72</v>
@@ -7232,13 +7250,13 @@
         <v>208</v>
       </c>
       <c r="I129" s="10" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="J129" s="10" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K129" s="10" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="L129" s="12"/>
       <c r="M129" s="13" t="s">
@@ -7250,16 +7268,16 @@
         <v>122</v>
       </c>
       <c r="C130" s="10" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D130" s="10" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E130" s="10" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F130" s="11" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G130" s="10" t="s">
         <v>236</v>
@@ -7268,53 +7286,49 @@
         <v>208</v>
       </c>
       <c r="I130" s="10" t="s">
-        <v>505</v>
+        <v>525</v>
       </c>
       <c r="J130" s="10" t="s">
-        <v>524</v>
-      </c>
-      <c r="K130" s="10" t="s">
-        <v>525</v>
-      </c>
+        <v>526</v>
+      </c>
+      <c r="K130" s="10"/>
       <c r="L130" s="12"/>
       <c r="M130" s="13" t="s">
         <v>506</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B131" s="9" t="n">
         <v>123</v>
       </c>
       <c r="C131" s="10" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D131" s="10" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F131" s="11" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G131" s="10" t="s">
-        <v>175</v>
+        <v>529</v>
       </c>
       <c r="H131" s="10" t="s">
-        <v>31</v>
+        <v>208</v>
       </c>
       <c r="I131" s="10" t="s">
-        <v>176</v>
+        <v>530</v>
       </c>
       <c r="J131" s="10" t="s">
-        <v>528</v>
-      </c>
-      <c r="K131" s="10" t="s">
-        <v>529</v>
-      </c>
+        <v>531</v>
+      </c>
+      <c r="K131" s="10"/>
       <c r="L131" s="12"/>
       <c r="M131" s="13" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7322,13 +7336,13 @@
         <v>124</v>
       </c>
       <c r="C132" s="10" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D132" s="10" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="E132" s="10" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="F132" s="11" t="s">
         <v>72</v>
@@ -7343,14 +7357,14 @@
         <v>256</v>
       </c>
       <c r="J132" s="10" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="K132" s="10" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="L132" s="12"/>
       <c r="M132" s="13" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7358,13 +7372,13 @@
         <v>125</v>
       </c>
       <c r="C133" s="10" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D133" s="10" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="F133" s="11" t="s">
         <v>72</v>
@@ -7382,11 +7396,11 @@
         <v>446</v>
       </c>
       <c r="K133" s="10" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="L133" s="12"/>
       <c r="M133" s="13" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7394,13 +7408,13 @@
         <v>126</v>
       </c>
       <c r="C134" s="10" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D134" s="10" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="E134" s="10" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="F134" s="11" t="s">
         <v>72</v>
@@ -7415,14 +7429,14 @@
         <v>256</v>
       </c>
       <c r="J134" s="10" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="K134" s="10" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="L134" s="12"/>
       <c r="M134" s="13" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7430,10 +7444,10 @@
         <v>127</v>
       </c>
       <c r="C135" s="10" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D135" s="10" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="E135" s="10" t="s">
         <v>59</v>
@@ -7451,12 +7465,12 @@
         <v>505</v>
       </c>
       <c r="J135" s="10" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="K135" s="10"/>
       <c r="L135" s="12"/>
       <c r="M135" s="13" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7464,13 +7478,13 @@
         <v>128</v>
       </c>
       <c r="C136" s="10" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D136" s="10" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E136" s="10" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F136" s="11" t="s">
         <v>86</v>
@@ -7488,7 +7502,7 @@
         <v>31</v>
       </c>
       <c r="K136" s="10" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="L136" s="12"/>
       <c r="M136" s="13" t="s">
@@ -7500,13 +7514,13 @@
         <v>129</v>
       </c>
       <c r="C137" s="10" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D137" s="10" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="E137" s="10" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="F137" s="11" t="s">
         <v>72</v>
@@ -7518,13 +7532,13 @@
         <v>208</v>
       </c>
       <c r="I137" s="10" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="J137" s="10" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="K137" s="10" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="L137" s="12"/>
       <c r="M137" s="13" t="s">
@@ -7536,122 +7550,124 @@
         <v>130</v>
       </c>
       <c r="C138" s="10" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="D138" s="10" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="E138" s="10" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="F138" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G138" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H138" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I138" s="10" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="J138" s="10" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="K138" s="10" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="L138" s="12"/>
       <c r="M138" s="13" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="139" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B139" s="9" t="n">
         <v>131</v>
       </c>
       <c r="C139" s="10" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="D139" s="10" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="E139" s="10" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="F139" s="11" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G139" s="10" t="s">
-        <v>559</v>
+        <v>202</v>
       </c>
       <c r="H139" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I139" s="10" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="J139" s="10" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="K139" s="10" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="L139" s="12"/>
       <c r="M139" s="13" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="140" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B140" s="9" t="n">
         <v>132</v>
       </c>
       <c r="C140" s="10" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="D140" s="10" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="E140" s="10" t="s">
-        <v>59</v>
+        <v>573</v>
       </c>
       <c r="F140" s="11" t="s">
         <v>29</v>
       </c>
       <c r="G140" s="10" t="s">
-        <v>559</v>
+        <v>202</v>
       </c>
       <c r="H140" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I140" s="10" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="J140" s="10" t="s">
-        <v>572</v>
-      </c>
-      <c r="K140" s="10"/>
+        <v>575</v>
+      </c>
+      <c r="K140" s="10" t="s">
+        <v>576</v>
+      </c>
       <c r="L140" s="12"/>
       <c r="M140" s="13" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="141" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B141" s="9" t="n">
         <v>133</v>
       </c>
       <c r="C141" s="10" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="D141" s="10" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="E141" s="10" t="s">
-        <v>31</v>
+        <v>578</v>
       </c>
       <c r="F141" s="11" t="s">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="G141" s="10" t="s">
         <v>202</v>
@@ -7660,51 +7676,49 @@
         <v>31</v>
       </c>
       <c r="I141" s="10" t="s">
-        <v>31</v>
+        <v>579</v>
       </c>
       <c r="J141" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="K141" s="10" t="s">
-        <v>358</v>
-      </c>
+        <v>580</v>
+      </c>
+      <c r="K141" s="10"/>
       <c r="L141" s="12"/>
       <c r="M141" s="13" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="142" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B142" s="9" t="n">
         <v>134</v>
       </c>
       <c r="C142" s="10" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="D142" s="10" t="s">
-        <v>574</v>
+        <v>581</v>
       </c>
       <c r="E142" s="10" t="s">
-        <v>59</v>
+        <v>582</v>
       </c>
       <c r="F142" s="11" t="s">
         <v>29</v>
       </c>
       <c r="G142" s="10" t="s">
-        <v>559</v>
+        <v>202</v>
       </c>
       <c r="H142" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I142" s="10" t="s">
-        <v>575</v>
+        <v>583</v>
       </c>
       <c r="J142" s="10" t="s">
-        <v>576</v>
+        <v>584</v>
       </c>
       <c r="K142" s="10"/>
       <c r="L142" s="12"/>
       <c r="M142" s="13" t="s">
-        <v>577</v>
+        <v>585</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7712,35 +7726,35 @@
         <v>135</v>
       </c>
       <c r="C143" s="10" t="s">
-        <v>578</v>
+        <v>586</v>
       </c>
       <c r="D143" s="10" t="s">
-        <v>579</v>
+        <v>587</v>
       </c>
       <c r="E143" s="10" t="s">
-        <v>580</v>
+        <v>588</v>
       </c>
       <c r="F143" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G143" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H143" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I143" s="10" t="s">
-        <v>581</v>
+        <v>589</v>
       </c>
       <c r="J143" s="10" t="s">
-        <v>582</v>
+        <v>590</v>
       </c>
       <c r="K143" s="10" t="s">
-        <v>583</v>
+        <v>591</v>
       </c>
       <c r="L143" s="12"/>
       <c r="M143" s="13" t="s">
-        <v>584</v>
+        <v>592</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7748,35 +7762,35 @@
         <v>136</v>
       </c>
       <c r="C144" s="10" t="s">
-        <v>578</v>
+        <v>586</v>
       </c>
       <c r="D144" s="10" t="s">
-        <v>585</v>
+        <v>593</v>
       </c>
       <c r="E144" s="10" t="s">
-        <v>586</v>
+        <v>594</v>
       </c>
       <c r="F144" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G144" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H144" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I144" s="10" t="s">
-        <v>581</v>
+        <v>589</v>
       </c>
       <c r="J144" s="10" t="s">
-        <v>587</v>
+        <v>595</v>
       </c>
       <c r="K144" s="10" t="s">
-        <v>588</v>
+        <v>596</v>
       </c>
       <c r="L144" s="12"/>
       <c r="M144" s="13" t="s">
-        <v>589</v>
+        <v>597</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7784,10 +7798,10 @@
         <v>137</v>
       </c>
       <c r="C145" s="10" t="s">
-        <v>590</v>
+        <v>598</v>
       </c>
       <c r="D145" s="10" t="s">
-        <v>591</v>
+        <v>599</v>
       </c>
       <c r="E145" s="10" t="s">
         <v>59</v>
@@ -7796,21 +7810,21 @@
         <v>29</v>
       </c>
       <c r="G145" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H145" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I145" s="10" t="s">
-        <v>592</v>
+        <v>600</v>
       </c>
       <c r="J145" s="10" t="s">
-        <v>593</v>
+        <v>601</v>
       </c>
       <c r="K145" s="10"/>
       <c r="L145" s="12"/>
       <c r="M145" s="13" t="s">
-        <v>594</v>
+        <v>602</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7818,10 +7832,10 @@
         <v>138</v>
       </c>
       <c r="C146" s="10" t="s">
-        <v>595</v>
+        <v>603</v>
       </c>
       <c r="D146" s="10" t="s">
-        <v>596</v>
+        <v>604</v>
       </c>
       <c r="E146" s="10" t="s">
         <v>59</v>
@@ -7830,21 +7844,21 @@
         <v>29</v>
       </c>
       <c r="G146" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H146" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I146" s="10" t="s">
-        <v>597</v>
+        <v>605</v>
       </c>
       <c r="J146" s="10" t="s">
-        <v>598</v>
+        <v>606</v>
       </c>
       <c r="K146" s="10"/>
       <c r="L146" s="12"/>
       <c r="M146" s="13" t="s">
-        <v>584</v>
+        <v>592</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7852,31 +7866,31 @@
         <v>139</v>
       </c>
       <c r="C147" s="10" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="D147" s="10" t="s">
-        <v>600</v>
+        <v>608</v>
       </c>
       <c r="E147" s="10" t="s">
-        <v>601</v>
+        <v>609</v>
       </c>
       <c r="F147" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G147" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H147" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I147" s="10" t="s">
-        <v>602</v>
+        <v>610</v>
       </c>
       <c r="J147" s="10" t="s">
-        <v>603</v>
+        <v>611</v>
       </c>
       <c r="K147" s="10" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="L147" s="12"/>
       <c r="M147" s="13" t="s">
@@ -7888,35 +7902,35 @@
         <v>140</v>
       </c>
       <c r="C148" s="10" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="D148" s="10" t="s">
-        <v>605</v>
+        <v>613</v>
       </c>
       <c r="E148" s="10" t="s">
-        <v>606</v>
+        <v>614</v>
       </c>
       <c r="F148" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G148" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H148" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I148" s="10" t="s">
-        <v>607</v>
+        <v>615</v>
       </c>
       <c r="J148" s="10" t="s">
-        <v>608</v>
+        <v>616</v>
       </c>
       <c r="K148" s="10" t="s">
-        <v>609</v>
+        <v>617</v>
       </c>
       <c r="L148" s="12"/>
       <c r="M148" s="13" t="s">
-        <v>610</v>
+        <v>618</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7924,19 +7938,19 @@
         <v>141</v>
       </c>
       <c r="C149" s="10" t="s">
-        <v>611</v>
+        <v>619</v>
       </c>
       <c r="D149" s="10" t="s">
-        <v>612</v>
+        <v>620</v>
       </c>
       <c r="E149" s="10" t="s">
-        <v>613</v>
+        <v>621</v>
       </c>
       <c r="F149" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G149" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H149" s="10" t="s">
         <v>31</v>
@@ -7948,7 +7962,7 @@
         <v>31</v>
       </c>
       <c r="K149" s="10" t="s">
-        <v>614</v>
+        <v>622</v>
       </c>
       <c r="L149" s="12"/>
       <c r="M149" s="13" t="s">
@@ -7960,10 +7974,10 @@
         <v>142</v>
       </c>
       <c r="C150" s="10" t="s">
-        <v>615</v>
+        <v>623</v>
       </c>
       <c r="D150" s="10" t="s">
-        <v>616</v>
+        <v>624</v>
       </c>
       <c r="E150" s="10" t="s">
         <v>59</v>
@@ -7972,21 +7986,21 @@
         <v>29</v>
       </c>
       <c r="G150" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H150" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I150" s="10" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="J150" s="10" t="s">
-        <v>618</v>
+        <v>626</v>
       </c>
       <c r="K150" s="10"/>
       <c r="L150" s="12"/>
       <c r="M150" s="13" t="s">
-        <v>619</v>
+        <v>627</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7994,35 +8008,35 @@
         <v>143</v>
       </c>
       <c r="C151" s="10" t="s">
-        <v>620</v>
+        <v>628</v>
       </c>
       <c r="D151" s="10" t="s">
-        <v>621</v>
+        <v>629</v>
       </c>
       <c r="E151" s="10" t="s">
-        <v>622</v>
+        <v>630</v>
       </c>
       <c r="F151" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G151" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H151" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I151" s="10" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="J151" s="10" t="s">
-        <v>623</v>
+        <v>631</v>
       </c>
       <c r="K151" s="10" t="s">
-        <v>624</v>
+        <v>632</v>
       </c>
       <c r="L151" s="12"/>
       <c r="M151" s="13" t="s">
-        <v>625</v>
+        <v>633</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8030,10 +8044,10 @@
         <v>144</v>
       </c>
       <c r="C152" s="10" t="s">
-        <v>626</v>
+        <v>634</v>
       </c>
       <c r="D152" s="10" t="s">
-        <v>627</v>
+        <v>635</v>
       </c>
       <c r="E152" s="10" t="s">
         <v>59</v>
@@ -8042,23 +8056,23 @@
         <v>29</v>
       </c>
       <c r="G152" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H152" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I152" s="10" t="s">
-        <v>628</v>
+        <v>636</v>
       </c>
       <c r="J152" s="10" t="s">
-        <v>629</v>
+        <v>637</v>
       </c>
       <c r="K152" s="10" t="s">
-        <v>630</v>
+        <v>638</v>
       </c>
       <c r="L152" s="12"/>
       <c r="M152" s="13" t="s">
-        <v>631</v>
+        <v>639</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8066,10 +8080,10 @@
         <v>145</v>
       </c>
       <c r="C153" s="10" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
       <c r="D153" s="10" t="s">
-        <v>633</v>
+        <v>641</v>
       </c>
       <c r="E153" s="10" t="s">
         <v>59</v>
@@ -8078,7 +8092,7 @@
         <v>29</v>
       </c>
       <c r="G153" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H153" s="10" t="s">
         <v>31</v>
@@ -8087,12 +8101,12 @@
         <v>217</v>
       </c>
       <c r="J153" s="10" t="s">
-        <v>634</v>
+        <v>642</v>
       </c>
       <c r="K153" s="10"/>
       <c r="L153" s="12"/>
       <c r="M153" s="13" t="s">
-        <v>635</v>
+        <v>643</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8100,13 +8114,13 @@
         <v>146</v>
       </c>
       <c r="C154" s="10" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
       <c r="D154" s="10" t="s">
-        <v>636</v>
+        <v>644</v>
       </c>
       <c r="E154" s="10" t="s">
-        <v>637</v>
+        <v>645</v>
       </c>
       <c r="F154" s="11" t="s">
         <v>72</v>
@@ -8121,14 +8135,14 @@
         <v>217</v>
       </c>
       <c r="J154" s="10" t="s">
-        <v>638</v>
+        <v>646</v>
       </c>
       <c r="K154" s="10" t="s">
-        <v>639</v>
+        <v>647</v>
       </c>
       <c r="L154" s="12"/>
       <c r="M154" s="13" t="s">
-        <v>619</v>
+        <v>627</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8136,10 +8150,10 @@
         <v>147</v>
       </c>
       <c r="C155" s="10" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
       <c r="D155" s="10" t="s">
-        <v>640</v>
+        <v>648</v>
       </c>
       <c r="E155" s="10" t="s">
         <v>31</v>
@@ -8148,7 +8162,7 @@
         <v>86</v>
       </c>
       <c r="G155" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="H155" s="10" t="s">
         <v>31</v>
@@ -8164,7 +8178,7 @@
       </c>
       <c r="L155" s="12"/>
       <c r="M155" s="13" t="s">
-        <v>641</v>
+        <v>649</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8172,10 +8186,10 @@
         <v>148</v>
       </c>
       <c r="C156" s="10" t="s">
-        <v>642</v>
+        <v>650</v>
       </c>
       <c r="D156" s="10" t="s">
-        <v>643</v>
+        <v>651</v>
       </c>
       <c r="E156" s="10" t="s">
         <v>59</v>
@@ -8190,17 +8204,17 @@
         <v>208</v>
       </c>
       <c r="I156" s="10" t="s">
-        <v>607</v>
+        <v>615</v>
       </c>
       <c r="J156" s="10" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="K156" s="10" t="s">
-        <v>645</v>
+        <v>653</v>
       </c>
       <c r="L156" s="12"/>
       <c r="M156" s="13" t="s">
-        <v>646</v>
+        <v>654</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8208,10 +8222,10 @@
         <v>149</v>
       </c>
       <c r="C157" s="10" t="s">
-        <v>642</v>
+        <v>650</v>
       </c>
       <c r="D157" s="10" t="s">
-        <v>647</v>
+        <v>655</v>
       </c>
       <c r="E157" s="10" t="s">
         <v>31</v>
@@ -8244,13 +8258,13 @@
         <v>150</v>
       </c>
       <c r="C158" s="10" t="s">
-        <v>642</v>
+        <v>650</v>
       </c>
       <c r="D158" s="10" t="s">
-        <v>648</v>
+        <v>656</v>
       </c>
       <c r="E158" s="10" t="s">
-        <v>649</v>
+        <v>657</v>
       </c>
       <c r="F158" s="11" t="s">
         <v>86</v>
@@ -8268,7 +8282,7 @@
         <v>31</v>
       </c>
       <c r="K158" s="10" t="s">
-        <v>650</v>
+        <v>658</v>
       </c>
       <c r="L158" s="12"/>
       <c r="M158" s="13" t="s">
@@ -8325,7 +8339,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="14" t="s">
-        <v>651</v>
+        <v>659</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8333,7 +8347,7 @@
         <v>15</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="D4" s="16" t="s">
         <v>29</v>
@@ -8348,7 +8362,7 @@
         <v>86</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8593,11 +8607,11 @@
       </c>
       <c r="D13" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B13,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E13" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B13,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B13,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -8609,7 +8623,7 @@
       </c>
       <c r="H13" s="19" t="n">
         <f aca="false">IF(C13&gt;0,D13/C13,0)</f>
-        <v>0.571428571428571</v>
+        <v>0.714285714285714</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9173,11 +9187,11 @@
       </c>
       <c r="D33" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B33,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E33" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B33,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B33,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -9185,16 +9199,16 @@
       </c>
       <c r="G33" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B33,'Master Requirements Tracker'!$F$9:$F$158,"Planned")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33" s="19" t="n">
         <f aca="false">IF(C33&gt;0,D33/C33,0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="17" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="C34" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B34)</f>
@@ -9202,11 +9216,11 @@
       </c>
       <c r="D34" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B34,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E34" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B34,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F34" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B34,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -9218,12 +9232,12 @@
       </c>
       <c r="H34" s="19" t="n">
         <f aca="false">IF(C34&gt;0,D34/C34,0)</f>
-        <v>0</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="17" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="C35" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B35)</f>
@@ -9252,7 +9266,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="17" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="C36" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B36)</f>
@@ -9281,7 +9295,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="17" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="C37" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B37)</f>
@@ -9310,7 +9324,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="17" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="C38" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B38)</f>
@@ -9339,7 +9353,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="17" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C39" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B39)</f>
@@ -9347,11 +9361,11 @@
       </c>
       <c r="D39" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B39,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E39" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B39,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B39,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -9359,16 +9373,16 @@
       </c>
       <c r="G39" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B39,'Master Requirements Tracker'!$F$9:$F$158,"Planned")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H39" s="19" t="n">
         <f aca="false">IF(C39&gt;0,D39/C39,0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="17" t="s">
-        <v>578</v>
+        <v>586</v>
       </c>
       <c r="C40" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B40)</f>
@@ -9397,7 +9411,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="17" t="s">
-        <v>590</v>
+        <v>598</v>
       </c>
       <c r="C41" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B41)</f>
@@ -9426,7 +9440,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="17" t="s">
-        <v>595</v>
+        <v>603</v>
       </c>
       <c r="C42" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B42)</f>
@@ -9455,7 +9469,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="17" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="C43" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B43)</f>
@@ -9484,7 +9498,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="17" t="s">
-        <v>611</v>
+        <v>619</v>
       </c>
       <c r="C44" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B44)</f>
@@ -9513,7 +9527,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="17" t="s">
-        <v>615</v>
+        <v>623</v>
       </c>
       <c r="C45" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B45)</f>
@@ -9542,7 +9556,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="17" t="s">
-        <v>620</v>
+        <v>628</v>
       </c>
       <c r="C46" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B46)</f>
@@ -9571,7 +9585,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="17" t="s">
-        <v>626</v>
+        <v>634</v>
       </c>
       <c r="C47" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B47)</f>
@@ -9600,7 +9614,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="17" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
       <c r="C48" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B48)</f>
@@ -9629,7 +9643,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="17" t="s">
-        <v>642</v>
+        <v>650</v>
       </c>
       <c r="C49" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B49)</f>
@@ -9658,7 +9672,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="20" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="C50" s="21" t="n">
         <f aca="false">SUM(C5:C49)</f>
@@ -9666,11 +9680,11 @@
       </c>
       <c r="D50" s="21" t="n">
         <f aca="false">SUM(D5:D49)</f>
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E50" s="21" t="n">
         <f aca="false">SUM(E5:E49)</f>
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F50" s="21" t="n">
         <f aca="false">SUM(F5:F49)</f>
@@ -9678,11 +9692,11 @@
       </c>
       <c r="G50" s="21" t="n">
         <f aca="false">SUM(G5:G49)</f>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H50" s="22" t="n">
         <f aca="false">IF(C50&gt;0,D50/C50,0)</f>
-        <v>0.613333333333333</v>
+        <v>0.66</v>
       </c>
     </row>
   </sheetData>
@@ -9713,18 +9727,18 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="14" t="s">
-        <v>654</v>
+        <v>662</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="23" t="s">
-        <v>655</v>
+        <v>663</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>656</v>
+        <v>664</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
       <c r="E4" s="23" t="s">
         <v>18</v>
@@ -9732,13 +9746,13 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="24" t="s">
-        <v>658</v>
+        <v>666</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>659</v>
+        <v>667</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="E5" s="25" t="s">
         <v>72</v>
@@ -9746,13 +9760,13 @@
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="24" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="E6" s="25" t="s">
         <v>72</v>
@@ -9760,13 +9774,13 @@
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="24" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="E7" s="25" t="s">
         <v>72</v>
@@ -9774,13 +9788,13 @@
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="24" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>668</v>
+        <v>676</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>669</v>
+        <v>677</v>
       </c>
       <c r="E8" s="25" t="s">
         <v>295</v>
@@ -9788,13 +9802,13 @@
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="24" t="s">
-        <v>670</v>
+        <v>678</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>671</v>
+        <v>679</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="E9" s="25" t="s">
         <v>72</v>
@@ -9802,13 +9816,13 @@
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="24" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>674</v>
+        <v>682</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>675</v>
+        <v>683</v>
       </c>
       <c r="E10" s="25" t="s">
         <v>86</v>
@@ -9816,13 +9830,13 @@
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="24" t="s">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>677</v>
+        <v>685</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="E11" s="25" t="s">
         <v>86</v>
@@ -9830,13 +9844,13 @@
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="24" t="s">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="E12" s="25" t="s">
         <v>86</v>
@@ -9888,15 +9902,15 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="14" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="26" t="s">
-        <v>683</v>
+        <v>691</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9904,7 +9918,7 @@
         <v>29</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9912,7 +9926,7 @@
         <v>72</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9920,7 +9934,7 @@
         <v>295</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9928,7 +9942,7 @@
         <v>86</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9936,7 +9950,7 @@
         <v>21</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>689</v>
+        <v>697</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9944,15 +9958,15 @@
         <v>22</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>690</v>
+        <v>698</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="26" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>692</v>
+        <v>700</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9960,15 +9974,15 @@
         <v>20</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>693</v>
+        <v>701</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="26" t="s">
-        <v>694</v>
+        <v>702</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>695</v>
+        <v>703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: referrals to Master — /r/CODE links, 90-day window, progress and rules
- /r/CODE (and ?deal=) website route; invite emails use the /r/ link
- All steps must finish within 90 days; late steps don't count; unfinished referrals expire
  (run from expire_reservations); new 'expired' status; admin Expired tab
- /users/me/referrals/ adds referral_link, reward_amount, window_days, summary and per-friend days_left
- Refer a Friend card: code + share link, Share a product, How it works, Earned/Pending/Invited,
  Step X of 4, expires in N days, Not eligible, Referral Rules sheet
- Tracker 102/150
</commit_message>
<xml_diff>
--- a/docs/client-requirements/Nibbl_Master_Requirements_Tracker.xlsx
+++ b/docs/client-requirements/Nibbl_Master_Requirements_Tracker.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1545" uniqueCount="704">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1542" uniqueCount="704">
   <si>
     <t xml:space="preserve">Nibbl AI — Master Requirements Tracker</t>
   </si>
@@ -1634,13 +1634,13 @@
     <t xml:space="preserve">Referral home, share link, share a product deal</t>
   </si>
   <si>
-    <t xml:space="preserve">Website invite card + Share this deal.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Copy the link.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Master link format is joinnibbl.com/r/CODE (we use ?ref=).</t>
+    <t xml:space="preserve">Code + copy, share sheet with joinnibbl.com/r/CODE, Share a product list (deal links carry the code), How it works.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → My Rewards → Refer a Friend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share the link; open it signed out.</t>
   </si>
   <si>
     <t xml:space="preserve">#40</t>
@@ -1649,22 +1649,22 @@
     <t xml:space="preserve">Qualification: join, claim, approved redemption, payout method, withdrawal — within 90 days</t>
   </si>
   <si>
-    <t xml:space="preserve">5-step qualification + review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">90-day completion window / expiry not built.</t>
+    <t xml:space="preserve">5-step qualification; only steps inside the 90-day window count; unfinished referrals expire (checked every 15 minutes).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backend; Admin → Referrals → Expired</t>
   </si>
   <si>
     <t xml:space="preserve">Referral progress (earned, pending, invited; step X of 4; expires in N days; not eligible) + rules sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Per-friend 5-step progress.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check a referral.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Totals, expiry countdown, 'not eligible' and rules sheet per mockup.</t>
+    <t xml:space="preserve">Earned / Pending / Invited totals, per-friend Step X of 4 + next step, Expires in N days, Earned / Not eligible, Referral Rules sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → My Rewards → My referrals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check a friend's progress.</t>
   </si>
   <si>
     <t xml:space="preserve">Shopper Restriction Messages</t>
@@ -2997,11 +2997,11 @@
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"Completed")</f>
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"In Progress")</f>
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"In Review")</f>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="H5" s="5" t="n">
         <f aca="false">IF(C5&gt;0,D5/C5,0)</f>
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7331,7 +7331,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B132" s="9" t="n">
         <v>124</v>
       </c>
@@ -7345,7 +7345,7 @@
         <v>535</v>
       </c>
       <c r="F132" s="11" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G132" s="10" t="s">
         <v>207</v>
@@ -7354,20 +7354,18 @@
         <v>208</v>
       </c>
       <c r="I132" s="10" t="s">
-        <v>256</v>
+        <v>536</v>
       </c>
       <c r="J132" s="10" t="s">
-        <v>536</v>
-      </c>
-      <c r="K132" s="10" t="s">
         <v>537</v>
       </c>
+      <c r="K132" s="10"/>
       <c r="L132" s="12"/>
       <c r="M132" s="13" t="s">
         <v>538</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B133" s="9" t="n">
         <v>125</v>
       </c>
@@ -7381,29 +7379,27 @@
         <v>540</v>
       </c>
       <c r="F133" s="11" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G133" s="10" t="s">
-        <v>175</v>
+        <v>216</v>
       </c>
       <c r="H133" s="10" t="s">
         <v>208</v>
       </c>
       <c r="I133" s="10" t="s">
-        <v>176</v>
+        <v>541</v>
       </c>
       <c r="J133" s="10" t="s">
         <v>446</v>
       </c>
-      <c r="K133" s="10" t="s">
-        <v>541</v>
-      </c>
+      <c r="K133" s="10"/>
       <c r="L133" s="12"/>
       <c r="M133" s="13" t="s">
         <v>538</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B134" s="9" t="n">
         <v>126</v>
       </c>
@@ -7417,23 +7413,21 @@
         <v>543</v>
       </c>
       <c r="F134" s="11" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G134" s="10" t="s">
-        <v>236</v>
+        <v>207</v>
       </c>
       <c r="H134" s="10" t="s">
         <v>208</v>
       </c>
       <c r="I134" s="10" t="s">
-        <v>256</v>
+        <v>544</v>
       </c>
       <c r="J134" s="10" t="s">
-        <v>544</v>
-      </c>
-      <c r="K134" s="10" t="s">
         <v>545</v>
       </c>
+      <c r="K134" s="10"/>
       <c r="L134" s="12"/>
       <c r="M134" s="13" t="s">
         <v>538</v>
@@ -9245,11 +9239,11 @@
       </c>
       <c r="D35" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B35,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E35" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B35,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F35" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B35,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -9261,7 +9255,7 @@
       </c>
       <c r="H35" s="19" t="n">
         <f aca="false">IF(C35&gt;0,D35/C35,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9680,11 +9674,11 @@
       </c>
       <c r="D50" s="21" t="n">
         <f aca="false">SUM(D5:D49)</f>
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E50" s="21" t="n">
         <f aca="false">SUM(E5:E49)</f>
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F50" s="21" t="n">
         <f aca="false">SUM(F5:F49)</f>
@@ -9696,7 +9690,7 @@
       </c>
       <c r="H50" s="22" t="n">
         <f aca="false">IF(C50&gt;0,D50/C50,0)</f>
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Customers to the Master: profile, cooldown removal, ban reason, table columns, 30-day receipt retention
- Customer Profile endpoint + page: opt-in badges, relationship with brand,
  Nibbl totals only, open claims, cooldowns with Remove (confirm + audit log),
  redemption history (full receipt 30 days, then matching line), activity
- Customer table: brand/site activity, open claims, cooldown days, status
- Ban with reason; banned shoppers get no review opportunities from the brand
- Receipt photo purge after 30 days (off until RECEIPT_IMAGE_PURGE_ENABLED)
</commit_message>
<xml_diff>
--- a/docs/client-requirements/Nibbl_Master_Requirements_Tracker.xlsx
+++ b/docs/client-requirements/Nibbl_Master_Requirements_Tracker.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1533" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1532" uniqueCount="720">
   <si>
     <t xml:space="preserve">Nibbl AI — Master Requirements Tracker</t>
   </si>
@@ -1229,13 +1229,10 @@
     <t xml:space="preserve">Table: brand activity, site activity, open claims, cooldowns, last active, status</t>
   </si>
   <si>
-    <t xml:space="preserve">Customer table.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open Customers.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site-activity and cooldown columns to match the mockup.</t>
+    <t xml:space="preserve">Columns per Master: Customer, Contact, Brand Activity (claims / rebates / reviews), Site Activity (total claims / % completion / reviews), Open Claims, Cooldowns (days left), Last Active, Status (Active / Banned), View. Tabs: All, Open Claim, Active Cooldown, Completed Rebate, Banned, Inactive.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open Customers; check each column and tab against a shopper with an open claim and a cooldown.</t>
   </si>
   <si>
     <t xml:space="preserve">Customer Profile</t>
@@ -1244,16 +1241,13 @@
     <t xml:space="preserve">Header (opt-in badges, status) + Ban Customer with reason</t>
   </si>
   <si>
-    <t xml:space="preserve">Suspend from brand exists.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customers → profile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suspend a customer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profile header/ban dialog per mockup.</t>
+    <t xml:space="preserve">Header: name, contact, customer since, last active, Nibbl Opt-In + brand Opt-In badges, Active/Banned. Ban modal with reason (suspicious activity, altered receipts, abuse, other); banned shoppers can't claim or get review opportunities from the brand; existing claims stay valid. Lift Ban.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers → View → Ban Customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ban with a reason; status shows Banned with the reason; Lift Ban restores it.</t>
   </si>
   <si>
     <t xml:space="preserve">#46</t>
@@ -1262,22 +1256,37 @@
     <t xml:space="preserve">Relationship with brand · Nibbl activity totals · Recent activity</t>
   </si>
   <si>
-    <t xml:space="preserve">Older profile layout.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open a profile.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rebuild to the Master layout.</t>
+    <t xml:space="preserve">Relationship tiles (claims, completed rebates, conversion, rewards, reviews, open claims); Nibbl totals only (claims, completion, reviews, rewards) — other brands' data never shown; recent activity timeline for this brand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers → View</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open a profile; totals match the shopper's history.</t>
   </si>
   <si>
     <t xml:space="preserve">Open claims · Cooldowns with Remove (confirmation + audit)</t>
   </si>
   <si>
+    <t xml:space="preserve">Open claims with days left. Rebate and review cooldowns with Remove → confirmation → cooldown cleared and an audit-log entry (who, when, which). Managers only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers → View → Cooldowns → Remove</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove a cooldown; the shopper can claim/review again; the audit log shows the removal.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Redemption history: full receipt 30 days, then matching line only</t>
   </si>
   <si>
-    <t xml:space="preserve">Receipt retention / cleanup rule not built.</t>
+    <t xml:space="preserve">Redemption history with View receipt + days left for 30 days; afterwards only the matching line item(s) are shown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers → View → Redemption History</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recent receipt shows View receipt; one older than 30 days shows Matching line only.</t>
   </si>
   <si>
     <t xml:space="preserve">Brand Wallet</t>
@@ -1610,7 +1619,7 @@
     <t xml:space="preserve">Withdraw a small amount.</t>
   </si>
   <si>
-    <t xml:space="preserve">Twilio approved — retest the SMS step on production, then Completed.</t>
+    <t xml:space="preserve">SMS verification works on production (12 Oct). Do one real website withdrawal with the SMS step, then Completed.</t>
   </si>
   <si>
     <t xml:space="preserve">'Additional review needed' popup; status stays Processing</t>
@@ -2012,6 +2021,18 @@
     <t xml:space="preserve">Receipt retention / cleanup (full receipt 30 days, then matching line only)</t>
   </si>
   <si>
+    <t xml:space="preserve">Scheduled job (every 15 min) deletes receipt images 30 days after submission (pending receipts are skipped) and records when; matching line items and receipt details stay.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backend job</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automated test: a 31-day-old receipt loses its image and keeps the matching line.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ships switched off in production (RECEIPT_IMAGE_PURGE_ENABLED) until the owner approves deleting existing receipt photos.</t>
+  </si>
+  <si>
     <t xml:space="preserve">System email via AWS SES with bounce / complaint handling</t>
   </si>
   <si>
@@ -2060,7 +2081,7 @@
     <t xml:space="preserve">Retest SMS-verified withdrawals; lock verified phones (change via admin + history)</t>
   </si>
   <si>
-    <t xml:space="preserve">Client: Twilio approved and ready for retesting</t>
+    <t xml:space="preserve">Twilio SMS verified on production 12 Oct 2026 (code sent to a Bangladesh number, delivered, approved). Remaining: one real website withdrawal with the SMS step</t>
   </si>
   <si>
     <t xml:space="preserve">Client — DNS</t>
@@ -2069,7 +2090,7 @@
     <t xml:space="preserve">Cloudflare access for www / brand / admin so the web apps can go live</t>
   </si>
   <si>
-    <t xml:space="preserve">Invite requested for syedriajul9624@gmail.com</t>
+    <t xml:space="preserve">Done — www / brand / admin.joinnibbl.com live with SSL on 11 Oct 2026</t>
   </si>
   <si>
     <t xml:space="preserve">AI service (Sakibur)</t>
@@ -2096,7 +2117,7 @@
     <t xml:space="preserve">System email from @joinnibbl.com + bounce/complaint handling</t>
   </si>
   <si>
-    <t xml:space="preserve">Done — production email switched to SES on 11 Oct 2026</t>
+    <t xml:space="preserve">Done — production email switched to SES on 11 Oct 2026 (per the client's 10 Oct credentials doc). Note: the Master says Klaviyo sends system emails — confirm SES is the long-term choice</t>
   </si>
   <si>
     <t xml:space="preserve">Client — Firebase</t>
@@ -2108,13 +2129,22 @@
     <t xml:space="preserve">Waiting on client setup</t>
   </si>
   <si>
-    <t xml:space="preserve">Client — Klaviyo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand + system SMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not integrated yet</t>
+    <t xml:space="preserve">Client — Klaviyo / SMS decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master Settings §3: 'Klaviyo will send Nibbl system emails and SMS messages' (Nibbl's internal Klaviyo account). Brand SMS toggles are stored but no SMS is sent yet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decision needed: Klaviyo access (private API key + SMS sender) as the Master says, or use the existing Twilio account for brand SMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client — FAQ content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand homepage 'Questions?' strip (Master mockup ④ only): Pricing / Review campaigns / Account &amp; billing / General FAQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No FAQ content in the Master — need questions/answers or a help-centre link; shown as labels until then</t>
   </si>
   <si>
     <t xml:space="preserve">How to Use This Tracker</t>
@@ -3015,11 +3045,11 @@
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"Completed")</f>
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"In Progress")</f>
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"In Review")</f>
@@ -3027,11 +3057,11 @@
       </c>
       <c r="G5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"Planned")</f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H5" s="5" t="n">
         <f aca="false">IF(C5&gt;0,D5/C5,0)</f>
-        <v>0.76</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6155,7 +6185,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B98" s="9" t="n">
         <v>90</v>
       </c>
@@ -6169,10 +6199,10 @@
         <v>400</v>
       </c>
       <c r="F98" s="11" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G98" s="10" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="H98" s="10" t="s">
         <v>31</v>
@@ -6183,101 +6213,95 @@
       <c r="J98" s="10" t="s">
         <v>401</v>
       </c>
-      <c r="K98" s="10" t="s">
-        <v>402</v>
-      </c>
+      <c r="K98" s="10"/>
       <c r="L98" s="12"/>
       <c r="M98" s="13" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B99" s="9" t="n">
         <v>91</v>
       </c>
       <c r="C99" s="10" t="s">
+        <v>402</v>
+      </c>
+      <c r="D99" s="10" t="s">
         <v>403</v>
       </c>
-      <c r="D99" s="10" t="s">
+      <c r="E99" s="10" t="s">
         <v>404</v>
       </c>
-      <c r="E99" s="10" t="s">
+      <c r="F99" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G99" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H99" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I99" s="10" t="s">
         <v>405</v>
       </c>
-      <c r="F99" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="G99" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H99" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I99" s="10" t="s">
+      <c r="J99" s="10" t="s">
         <v>406</v>
       </c>
-      <c r="J99" s="10" t="s">
-        <v>407</v>
-      </c>
-      <c r="K99" s="10" t="s">
-        <v>408</v>
-      </c>
+      <c r="K99" s="10"/>
       <c r="L99" s="12"/>
       <c r="M99" s="13" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B100" s="9" t="n">
         <v>92</v>
       </c>
       <c r="C100" s="10" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D100" s="10" t="s">
+        <v>408</v>
+      </c>
+      <c r="E100" s="10" t="s">
+        <v>409</v>
+      </c>
+      <c r="F100" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G100" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H100" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I100" s="10" t="s">
         <v>410</v>
       </c>
-      <c r="E100" s="10" t="s">
+      <c r="J100" s="10" t="s">
         <v>411</v>
       </c>
-      <c r="F100" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="G100" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H100" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I100" s="10" t="s">
-        <v>406</v>
-      </c>
-      <c r="J100" s="10" t="s">
-        <v>412</v>
-      </c>
-      <c r="K100" s="10" t="s">
-        <v>413</v>
-      </c>
+      <c r="K100" s="10"/>
       <c r="L100" s="12"/>
       <c r="M100" s="13" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B101" s="9" t="n">
         <v>93</v>
       </c>
       <c r="C101" s="10" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D101" s="10" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>31</v>
+        <v>413</v>
       </c>
       <c r="F101" s="11" t="s">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="G101" s="10" t="s">
         <v>51</v>
@@ -6286,34 +6310,32 @@
         <v>31</v>
       </c>
       <c r="I101" s="10" t="s">
-        <v>31</v>
+        <v>414</v>
       </c>
       <c r="J101" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="K101" s="10" t="s">
-        <v>361</v>
-      </c>
+        <v>415</v>
+      </c>
+      <c r="K101" s="10"/>
       <c r="L101" s="12"/>
       <c r="M101" s="13" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B102" s="9" t="n">
         <v>94</v>
       </c>
       <c r="C102" s="10" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D102" s="10" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="E102" s="10" t="s">
-        <v>31</v>
+        <v>417</v>
       </c>
       <c r="F102" s="11" t="s">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="G102" s="10" t="s">
         <v>51</v>
@@ -6322,14 +6344,12 @@
         <v>31</v>
       </c>
       <c r="I102" s="10" t="s">
-        <v>31</v>
+        <v>418</v>
       </c>
       <c r="J102" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="K102" s="10" t="s">
-        <v>416</v>
-      </c>
+        <v>419</v>
+      </c>
+      <c r="K102" s="10"/>
       <c r="L102" s="12"/>
       <c r="M102" s="13" t="s">
         <v>398</v>
@@ -6340,10 +6360,10 @@
         <v>95</v>
       </c>
       <c r="C103" s="10" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D103" s="10" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>59</v>
@@ -6358,15 +6378,15 @@
         <v>31</v>
       </c>
       <c r="I103" s="10" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="J103" s="10" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="K103" s="10"/>
       <c r="L103" s="12"/>
       <c r="M103" s="13" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6374,10 +6394,10 @@
         <v>96</v>
       </c>
       <c r="C104" s="10" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D104" s="10" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="E104" s="10" t="s">
         <v>59</v>
@@ -6392,15 +6412,15 @@
         <v>31</v>
       </c>
       <c r="I104" s="10" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="J104" s="10" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="K104" s="10"/>
       <c r="L104" s="12"/>
       <c r="M104" s="13" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6408,10 +6428,10 @@
         <v>97</v>
       </c>
       <c r="C105" s="10" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D105" s="10" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>59</v>
@@ -6426,17 +6446,17 @@
         <v>31</v>
       </c>
       <c r="I105" s="10" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="J105" s="10" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="K105" s="10" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="L105" s="12"/>
       <c r="M105" s="13" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6444,10 +6464,10 @@
         <v>98</v>
       </c>
       <c r="C106" s="10" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D106" s="10" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="E106" s="10" t="s">
         <v>59</v>
@@ -6462,15 +6482,15 @@
         <v>31</v>
       </c>
       <c r="I106" s="10" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="J106" s="10" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="K106" s="10"/>
       <c r="L106" s="12"/>
       <c r="M106" s="13" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6478,31 +6498,31 @@
         <v>99</v>
       </c>
       <c r="C107" s="10" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D107" s="10" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="F107" s="11" t="s">
         <v>29</v>
       </c>
       <c r="G107" s="10" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="H107" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I107" s="10" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="J107" s="10" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="K107" s="10" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="L107" s="12"/>
       <c r="M107" s="13" t="s">
@@ -6514,10 +6534,10 @@
         <v>100</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="D108" s="10" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="E108" s="10" t="s">
         <v>59</v>
@@ -6532,15 +6552,15 @@
         <v>31</v>
       </c>
       <c r="I108" s="10" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="J108" s="10" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="K108" s="10"/>
       <c r="L108" s="12"/>
       <c r="M108" s="13" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6548,13 +6568,13 @@
         <v>101</v>
       </c>
       <c r="C109" s="10" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="D109" s="10" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="F109" s="11" t="s">
         <v>29</v>
@@ -6566,10 +6586,10 @@
         <v>31</v>
       </c>
       <c r="I109" s="10" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="J109" s="10" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="K109" s="10"/>
       <c r="L109" s="12"/>
@@ -6582,13 +6602,13 @@
         <v>102</v>
       </c>
       <c r="C110" s="10" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="D110" s="10" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="E110" s="10" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="F110" s="11" t="s">
         <v>29</v>
@@ -6603,12 +6623,12 @@
         <v>176</v>
       </c>
       <c r="J110" s="10" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="K110" s="10"/>
       <c r="L110" s="12"/>
       <c r="M110" s="13" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6616,10 +6636,10 @@
         <v>103</v>
       </c>
       <c r="C111" s="10" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D111" s="10" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="E111" s="10" t="s">
         <v>59</v>
@@ -6634,15 +6654,15 @@
         <v>31</v>
       </c>
       <c r="I111" s="10" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="J111" s="10" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="K111" s="10"/>
       <c r="L111" s="12"/>
       <c r="M111" s="13" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6650,10 +6670,10 @@
         <v>104</v>
       </c>
       <c r="C112" s="10" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D112" s="10" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="E112" s="10" t="s">
         <v>59</v>
@@ -6668,15 +6688,15 @@
         <v>31</v>
       </c>
       <c r="I112" s="10" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="J112" s="10" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="K112" s="10"/>
       <c r="L112" s="12"/>
       <c r="M112" s="13" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6684,13 +6704,13 @@
         <v>105</v>
       </c>
       <c r="C113" s="10" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D113" s="10" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="F113" s="11" t="s">
         <v>72</v>
@@ -6702,17 +6722,17 @@
         <v>31</v>
       </c>
       <c r="I113" s="10" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="J113" s="10" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="K113" s="10" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="L113" s="12"/>
       <c r="M113" s="13" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6720,10 +6740,10 @@
         <v>106</v>
       </c>
       <c r="C114" s="10" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D114" s="10" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="E114" s="10" t="s">
         <v>59</v>
@@ -6738,10 +6758,10 @@
         <v>31</v>
       </c>
       <c r="I114" s="10" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="J114" s="10" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="K114" s="10"/>
       <c r="L114" s="12"/>
@@ -6754,13 +6774,13 @@
         <v>107</v>
       </c>
       <c r="C115" s="10" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D115" s="10" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="E115" s="10" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="F115" s="11" t="s">
         <v>29</v>
@@ -6772,15 +6792,15 @@
         <v>31</v>
       </c>
       <c r="I115" s="10" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="J115" s="10" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="K115" s="10"/>
       <c r="L115" s="12"/>
       <c r="M115" s="13" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6788,10 +6808,10 @@
         <v>108</v>
       </c>
       <c r="C116" s="10" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D116" s="10" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="E116" s="10" t="s">
         <v>59</v>
@@ -6806,15 +6826,15 @@
         <v>31</v>
       </c>
       <c r="I116" s="10" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="J116" s="10" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="K116" s="10"/>
       <c r="L116" s="12"/>
       <c r="M116" s="13" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6822,10 +6842,10 @@
         <v>109</v>
       </c>
       <c r="C117" s="10" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="D117" s="10" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="E117" s="10" t="s">
         <v>59</v>
@@ -6840,15 +6860,15 @@
         <v>31</v>
       </c>
       <c r="I117" s="10" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="J117" s="10" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="K117" s="10"/>
       <c r="L117" s="12"/>
       <c r="M117" s="13" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6856,13 +6876,13 @@
         <v>110</v>
       </c>
       <c r="C118" s="10" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="D118" s="10" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="E118" s="10" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="F118" s="11" t="s">
         <v>29</v>
@@ -6874,7 +6894,7 @@
         <v>31</v>
       </c>
       <c r="I118" s="10" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="J118" s="10" t="s">
         <v>229</v>
@@ -6882,7 +6902,7 @@
       <c r="K118" s="10"/>
       <c r="L118" s="12"/>
       <c r="M118" s="13" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6890,13 +6910,13 @@
         <v>111</v>
       </c>
       <c r="C119" s="10" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="D119" s="10" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="E119" s="10" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="F119" s="11" t="s">
         <v>29</v>
@@ -6908,17 +6928,17 @@
         <v>31</v>
       </c>
       <c r="I119" s="10" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J119" s="10" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="K119" s="10" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="L119" s="12"/>
       <c r="M119" s="13" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6926,13 +6946,13 @@
         <v>112</v>
       </c>
       <c r="C120" s="10" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="D120" s="10" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="E120" s="10" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="F120" s="11" t="s">
         <v>29</v>
@@ -6944,15 +6964,15 @@
         <v>31</v>
       </c>
       <c r="I120" s="10" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="J120" s="10" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="K120" s="10"/>
       <c r="L120" s="12"/>
       <c r="M120" s="13" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6960,13 +6980,13 @@
         <v>113</v>
       </c>
       <c r="C121" s="10" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="D121" s="10" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="E121" s="10" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="F121" s="11" t="s">
         <v>29</v>
@@ -6978,15 +6998,15 @@
         <v>31</v>
       </c>
       <c r="I121" s="10" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="J121" s="10" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="K121" s="10"/>
       <c r="L121" s="12"/>
       <c r="M121" s="13" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6994,13 +7014,13 @@
         <v>114</v>
       </c>
       <c r="C122" s="10" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="D122" s="10" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="E122" s="10" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="F122" s="11" t="s">
         <v>29</v>
@@ -7012,17 +7032,17 @@
         <v>31</v>
       </c>
       <c r="I122" s="10" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="J122" s="10" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="K122" s="10" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="L122" s="12"/>
       <c r="M122" s="13" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7030,13 +7050,13 @@
         <v>115</v>
       </c>
       <c r="C123" s="10" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="D123" s="10" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="E123" s="10" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="F123" s="11" t="s">
         <v>29</v>
@@ -7048,15 +7068,15 @@
         <v>31</v>
       </c>
       <c r="I123" s="10" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="J123" s="10" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="K123" s="10"/>
       <c r="L123" s="12"/>
       <c r="M123" s="13" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7064,13 +7084,13 @@
         <v>116</v>
       </c>
       <c r="C124" s="10" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="D124" s="10" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="E124" s="10" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="F124" s="11" t="s">
         <v>29</v>
@@ -7082,15 +7102,15 @@
         <v>31</v>
       </c>
       <c r="I124" s="10" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="J124" s="10" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="K124" s="10"/>
       <c r="L124" s="12"/>
       <c r="M124" s="13" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7098,10 +7118,10 @@
         <v>117</v>
       </c>
       <c r="C125" s="10" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D125" s="10" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="E125" s="10" t="s">
         <v>59</v>
@@ -7116,15 +7136,15 @@
         <v>208</v>
       </c>
       <c r="I125" s="10" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="J125" s="10" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="K125" s="10"/>
       <c r="L125" s="12"/>
       <c r="M125" s="13" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7132,13 +7152,13 @@
         <v>118</v>
       </c>
       <c r="C126" s="10" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D126" s="10" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="E126" s="10" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="F126" s="11" t="s">
         <v>29</v>
@@ -7150,7 +7170,7 @@
         <v>208</v>
       </c>
       <c r="I126" s="10" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="J126" s="10" t="s">
         <v>115</v>
@@ -7158,7 +7178,7 @@
       <c r="K126" s="10"/>
       <c r="L126" s="12"/>
       <c r="M126" s="13" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7166,13 +7186,13 @@
         <v>119</v>
       </c>
       <c r="C127" s="10" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D127" s="10" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="E127" s="10" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="F127" s="11" t="s">
         <v>29</v>
@@ -7184,15 +7204,15 @@
         <v>208</v>
       </c>
       <c r="I127" s="10" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="J127" s="10" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="K127" s="10"/>
       <c r="L127" s="12"/>
       <c r="M127" s="13" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7200,10 +7220,10 @@
         <v>120</v>
       </c>
       <c r="C128" s="10" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D128" s="10" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="E128" s="10" t="s">
         <v>59</v>
@@ -7218,15 +7238,15 @@
         <v>208</v>
       </c>
       <c r="I128" s="10" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="J128" s="10" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="K128" s="10"/>
       <c r="L128" s="12"/>
       <c r="M128" s="13" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7234,13 +7254,13 @@
         <v>121</v>
       </c>
       <c r="C129" s="10" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="D129" s="10" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="E129" s="10" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="F129" s="11" t="s">
         <v>72</v>
@@ -7252,17 +7272,17 @@
         <v>208</v>
       </c>
       <c r="I129" s="10" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="J129" s="10" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="K129" s="10" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="L129" s="12"/>
       <c r="M129" s="13" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7270,13 +7290,13 @@
         <v>122</v>
       </c>
       <c r="C130" s="10" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="D130" s="10" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="E130" s="10" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="F130" s="11" t="s">
         <v>29</v>
@@ -7288,15 +7308,15 @@
         <v>208</v>
       </c>
       <c r="I130" s="10" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="J130" s="10" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="K130" s="10"/>
       <c r="L130" s="12"/>
       <c r="M130" s="13" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7304,33 +7324,33 @@
         <v>123</v>
       </c>
       <c r="C131" s="10" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="D131" s="10" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="F131" s="11" t="s">
         <v>29</v>
       </c>
       <c r="G131" s="10" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="H131" s="10" t="s">
         <v>208</v>
       </c>
       <c r="I131" s="10" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="J131" s="10" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="K131" s="10"/>
       <c r="L131" s="12"/>
       <c r="M131" s="13" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7338,13 +7358,13 @@
         <v>124</v>
       </c>
       <c r="C132" s="10" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="D132" s="10" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="E132" s="10" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="F132" s="11" t="s">
         <v>29</v>
@@ -7356,15 +7376,15 @@
         <v>208</v>
       </c>
       <c r="I132" s="10" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="J132" s="10" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="K132" s="10"/>
       <c r="L132" s="12"/>
       <c r="M132" s="13" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7372,13 +7392,13 @@
         <v>125</v>
       </c>
       <c r="C133" s="10" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="D133" s="10" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="F133" s="11" t="s">
         <v>29</v>
@@ -7390,15 +7410,15 @@
         <v>208</v>
       </c>
       <c r="I133" s="10" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="J133" s="10" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="K133" s="10"/>
       <c r="L133" s="12"/>
       <c r="M133" s="13" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7406,13 +7426,13 @@
         <v>126</v>
       </c>
       <c r="C134" s="10" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="D134" s="10" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="E134" s="10" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="F134" s="11" t="s">
         <v>29</v>
@@ -7424,15 +7444,15 @@
         <v>208</v>
       </c>
       <c r="I134" s="10" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="J134" s="10" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="K134" s="10"/>
       <c r="L134" s="12"/>
       <c r="M134" s="13" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7440,10 +7460,10 @@
         <v>127</v>
       </c>
       <c r="C135" s="10" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="D135" s="10" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="E135" s="10" t="s">
         <v>59</v>
@@ -7458,15 +7478,15 @@
         <v>208</v>
       </c>
       <c r="I135" s="10" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="J135" s="10" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="K135" s="10"/>
       <c r="L135" s="12"/>
       <c r="M135" s="13" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7474,13 +7494,13 @@
         <v>128</v>
       </c>
       <c r="C136" s="10" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="D136" s="10" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="E136" s="10" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="F136" s="11" t="s">
         <v>86</v>
@@ -7498,7 +7518,7 @@
         <v>31</v>
       </c>
       <c r="K136" s="10" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="L136" s="12"/>
       <c r="M136" s="13" t="s">
@@ -7510,13 +7530,13 @@
         <v>129</v>
       </c>
       <c r="C137" s="10" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="D137" s="10" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="E137" s="10" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="F137" s="11" t="s">
         <v>72</v>
@@ -7528,17 +7548,17 @@
         <v>208</v>
       </c>
       <c r="I137" s="10" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="J137" s="10" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="K137" s="10" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="L137" s="12"/>
       <c r="M137" s="13" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7546,35 +7566,35 @@
         <v>130</v>
       </c>
       <c r="C138" s="10" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="D138" s="10" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="E138" s="10" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="F138" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G138" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H138" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I138" s="10" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="J138" s="10" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K138" s="10" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L138" s="12"/>
       <c r="M138" s="13" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7582,13 +7602,13 @@
         <v>131</v>
       </c>
       <c r="C139" s="10" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D139" s="10" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="E139" s="10" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="F139" s="11" t="s">
         <v>29</v>
@@ -7600,17 +7620,17 @@
         <v>31</v>
       </c>
       <c r="I139" s="10" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="J139" s="10" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="K139" s="10" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="L139" s="12"/>
       <c r="M139" s="13" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7618,13 +7638,13 @@
         <v>132</v>
       </c>
       <c r="C140" s="10" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D140" s="10" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="E140" s="10" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="F140" s="11" t="s">
         <v>29</v>
@@ -7636,17 +7656,17 @@
         <v>31</v>
       </c>
       <c r="I140" s="10" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="J140" s="10" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="K140" s="10" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="L140" s="12"/>
       <c r="M140" s="13" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7654,13 +7674,13 @@
         <v>133</v>
       </c>
       <c r="C141" s="10" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D141" s="10" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E141" s="10" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="F141" s="11" t="s">
         <v>29</v>
@@ -7672,15 +7692,15 @@
         <v>31</v>
       </c>
       <c r="I141" s="10" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="J141" s="10" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="K141" s="10"/>
       <c r="L141" s="12"/>
       <c r="M141" s="13" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7688,13 +7708,13 @@
         <v>134</v>
       </c>
       <c r="C142" s="10" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D142" s="10" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="E142" s="10" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="F142" s="11" t="s">
         <v>29</v>
@@ -7706,15 +7726,15 @@
         <v>31</v>
       </c>
       <c r="I142" s="10" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="J142" s="10" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="K142" s="10"/>
       <c r="L142" s="12"/>
       <c r="M142" s="13" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7722,35 +7742,35 @@
         <v>135</v>
       </c>
       <c r="C143" s="10" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="D143" s="10" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="E143" s="10" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="F143" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G143" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H143" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I143" s="10" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="J143" s="10" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="K143" s="10" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="L143" s="12"/>
       <c r="M143" s="13" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7758,35 +7778,35 @@
         <v>136</v>
       </c>
       <c r="C144" s="10" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="D144" s="10" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="E144" s="10" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="F144" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G144" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H144" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I144" s="10" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="J144" s="10" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="K144" s="10" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="L144" s="12"/>
       <c r="M144" s="13" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7794,10 +7814,10 @@
         <v>137</v>
       </c>
       <c r="C145" s="10" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="D145" s="10" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="E145" s="10" t="s">
         <v>59</v>
@@ -7806,21 +7826,21 @@
         <v>29</v>
       </c>
       <c r="G145" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H145" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I145" s="10" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="J145" s="10" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="K145" s="10"/>
       <c r="L145" s="12"/>
       <c r="M145" s="13" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7828,10 +7848,10 @@
         <v>138</v>
       </c>
       <c r="C146" s="10" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="D146" s="10" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="E146" s="10" t="s">
         <v>59</v>
@@ -7840,21 +7860,21 @@
         <v>29</v>
       </c>
       <c r="G146" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H146" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I146" s="10" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="J146" s="10" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="K146" s="10"/>
       <c r="L146" s="12"/>
       <c r="M146" s="13" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7862,35 +7882,35 @@
         <v>139</v>
       </c>
       <c r="C147" s="10" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="D147" s="10" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="E147" s="10" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="F147" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G147" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H147" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I147" s="10" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="J147" s="10" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="K147" s="10" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="L147" s="12"/>
       <c r="M147" s="13" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7898,35 +7918,35 @@
         <v>140</v>
       </c>
       <c r="C148" s="10" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="D148" s="10" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="E148" s="10" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="F148" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G148" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H148" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I148" s="10" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="J148" s="10" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="K148" s="10" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="L148" s="12"/>
       <c r="M148" s="13" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7934,19 +7954,19 @@
         <v>141</v>
       </c>
       <c r="C149" s="10" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="D149" s="10" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="E149" s="10" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="F149" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G149" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H149" s="10" t="s">
         <v>31</v>
@@ -7958,11 +7978,11 @@
         <v>31</v>
       </c>
       <c r="K149" s="10" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="L149" s="12"/>
       <c r="M149" s="13" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7970,10 +7990,10 @@
         <v>142</v>
       </c>
       <c r="C150" s="10" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="D150" s="10" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="E150" s="10" t="s">
         <v>59</v>
@@ -7982,21 +8002,21 @@
         <v>29</v>
       </c>
       <c r="G150" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H150" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I150" s="10" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="J150" s="10" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="K150" s="10"/>
       <c r="L150" s="12"/>
       <c r="M150" s="13" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8004,35 +8024,35 @@
         <v>143</v>
       </c>
       <c r="C151" s="10" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="D151" s="10" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="E151" s="10" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="F151" s="11" t="s">
         <v>72</v>
       </c>
       <c r="G151" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H151" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I151" s="10" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="J151" s="10" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="K151" s="10" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="L151" s="12"/>
       <c r="M151" s="13" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8040,10 +8060,10 @@
         <v>144</v>
       </c>
       <c r="C152" s="10" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="D152" s="10" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="E152" s="10" t="s">
         <v>59</v>
@@ -8052,23 +8072,23 @@
         <v>29</v>
       </c>
       <c r="G152" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H152" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I152" s="10" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="J152" s="10" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="K152" s="10" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="L152" s="12"/>
       <c r="M152" s="13" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8076,10 +8096,10 @@
         <v>145</v>
       </c>
       <c r="C153" s="10" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="D153" s="10" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="E153" s="10" t="s">
         <v>59</v>
@@ -8088,7 +8108,7 @@
         <v>29</v>
       </c>
       <c r="G153" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H153" s="10" t="s">
         <v>31</v>
@@ -8097,12 +8117,12 @@
         <v>217</v>
       </c>
       <c r="J153" s="10" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="K153" s="10"/>
       <c r="L153" s="12"/>
       <c r="M153" s="13" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8110,13 +8130,13 @@
         <v>146</v>
       </c>
       <c r="C154" s="10" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="D154" s="10" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="E154" s="10" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="F154" s="11" t="s">
         <v>72</v>
@@ -8131,14 +8151,14 @@
         <v>217</v>
       </c>
       <c r="J154" s="10" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="K154" s="10" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="L154" s="12"/>
       <c r="M154" s="13" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8146,10 +8166,10 @@
         <v>147</v>
       </c>
       <c r="C155" s="10" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="D155" s="10" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
       <c r="E155" s="10" t="s">
         <v>31</v>
@@ -8158,7 +8178,7 @@
         <v>86</v>
       </c>
       <c r="G155" s="10" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="H155" s="10" t="s">
         <v>31</v>
@@ -8174,7 +8194,7 @@
       </c>
       <c r="L155" s="12"/>
       <c r="M155" s="13" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8182,10 +8202,10 @@
         <v>148</v>
       </c>
       <c r="C156" s="10" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="D156" s="10" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="E156" s="10" t="s">
         <v>59</v>
@@ -8200,34 +8220,34 @@
         <v>208</v>
       </c>
       <c r="I156" s="10" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="J156" s="10" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="K156" s="10" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="L156" s="12"/>
       <c r="M156" s="13" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="157" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B157" s="9" t="n">
         <v>149</v>
       </c>
       <c r="C157" s="10" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="D157" s="10" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="E157" s="10" t="s">
-        <v>31</v>
+        <v>664</v>
       </c>
       <c r="F157" s="11" t="s">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="G157" s="10" t="s">
         <v>175</v>
@@ -8236,13 +8256,13 @@
         <v>31</v>
       </c>
       <c r="I157" s="10" t="s">
-        <v>31</v>
+        <v>665</v>
       </c>
       <c r="J157" s="10" t="s">
-        <v>31</v>
+        <v>666</v>
       </c>
       <c r="K157" s="10" t="s">
-        <v>361</v>
+        <v>667</v>
       </c>
       <c r="L157" s="12"/>
       <c r="M157" s="13" t="s">
@@ -8254,13 +8274,13 @@
         <v>150</v>
       </c>
       <c r="C158" s="10" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="D158" s="10" t="s">
-        <v>661</v>
+        <v>668</v>
       </c>
       <c r="E158" s="10" t="s">
-        <v>662</v>
+        <v>669</v>
       </c>
       <c r="F158" s="11" t="s">
         <v>29</v>
@@ -8272,10 +8292,10 @@
         <v>31</v>
       </c>
       <c r="I158" s="10" t="s">
-        <v>663</v>
+        <v>670</v>
       </c>
       <c r="J158" s="10" t="s">
-        <v>664</v>
+        <v>671</v>
       </c>
       <c r="K158" s="10"/>
       <c r="L158" s="12"/>
@@ -8333,7 +8353,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="14" t="s">
-        <v>665</v>
+        <v>672</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8341,7 +8361,7 @@
         <v>15</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>666</v>
+        <v>673</v>
       </c>
       <c r="D4" s="16" t="s">
         <v>29</v>
@@ -8356,7 +8376,7 @@
         <v>86</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>667</v>
+        <v>674</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8978,11 +8998,11 @@
       </c>
       <c r="D26" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B26,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B26,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B26,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -8994,12 +9014,12 @@
       </c>
       <c r="H26" s="19" t="n">
         <f aca="false">IF(C26&gt;0,D26/C26,0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="17" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C27" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B27)</f>
@@ -9007,11 +9027,11 @@
       </c>
       <c r="D27" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B27,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E27" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B27,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F27" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B27,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -9019,16 +9039,16 @@
       </c>
       <c r="G27" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B27,'Master Requirements Tracker'!$F$9:$F$158,"Planned")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H27" s="19" t="n">
         <f aca="false">IF(C27&gt;0,D27/C27,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="17" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="C28" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B28)</f>
@@ -9057,7 +9077,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="17" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="C29" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B29)</f>
@@ -9086,7 +9106,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="17" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="C30" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B30)</f>
@@ -9115,7 +9135,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="17" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="C31" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B31)</f>
@@ -9144,7 +9164,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="17" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="C32" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B32)</f>
@@ -9173,7 +9193,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="17" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="C33" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B33)</f>
@@ -9202,7 +9222,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="17" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="C34" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B34)</f>
@@ -9231,7 +9251,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="17" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="C35" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B35)</f>
@@ -9260,7 +9280,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="17" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="C36" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B36)</f>
@@ -9289,7 +9309,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="17" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="C37" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B37)</f>
@@ -9318,7 +9338,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="17" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="C38" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B38)</f>
@@ -9347,7 +9367,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="17" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="C39" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B39)</f>
@@ -9376,7 +9396,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="17" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C40" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B40)</f>
@@ -9405,7 +9425,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="17" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="C41" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B41)</f>
@@ -9434,7 +9454,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="17" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="C42" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B42)</f>
@@ -9463,7 +9483,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="17" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="C43" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B43)</f>
@@ -9492,7 +9512,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="17" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="C44" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B44)</f>
@@ -9521,7 +9541,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="17" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="C45" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B45)</f>
@@ -9550,7 +9570,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="17" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="C46" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B46)</f>
@@ -9579,7 +9599,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="17" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="C47" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B47)</f>
@@ -9608,7 +9628,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="17" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="C48" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B48)</f>
@@ -9637,7 +9657,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="17" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="C49" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B49)</f>
@@ -9645,7 +9665,7 @@
       </c>
       <c r="D49" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B49,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E49" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B49,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
@@ -9657,16 +9677,16 @@
       </c>
       <c r="G49" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B49,'Master Requirements Tracker'!$F$9:$F$158,"Planned")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H49" s="19" t="n">
         <f aca="false">IF(C49&gt;0,D49/C49,0)</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="20" t="s">
-        <v>666</v>
+        <v>673</v>
       </c>
       <c r="C50" s="21" t="n">
         <f aca="false">SUM(C5:C49)</f>
@@ -9674,11 +9694,11 @@
       </c>
       <c r="D50" s="21" t="n">
         <f aca="false">SUM(D5:D49)</f>
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="E50" s="21" t="n">
         <f aca="false">SUM(E5:E49)</f>
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F50" s="21" t="n">
         <f aca="false">SUM(F5:F49)</f>
@@ -9686,11 +9706,11 @@
       </c>
       <c r="G50" s="21" t="n">
         <f aca="false">SUM(G5:G49)</f>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H50" s="22" t="n">
         <f aca="false">IF(C50&gt;0,D50/C50,0)</f>
-        <v>0.76</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -9709,7 +9729,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:E12"/>
+  <dimension ref="B2:E13"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.75"/>
@@ -9721,18 +9741,18 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="14" t="s">
-        <v>668</v>
+        <v>675</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="23" t="s">
-        <v>669</v>
+        <v>676</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>670</v>
+        <v>677</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>671</v>
+        <v>678</v>
       </c>
       <c r="E4" s="23" t="s">
         <v>18</v>
@@ -9740,13 +9760,13 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="24" t="s">
-        <v>672</v>
+        <v>679</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>673</v>
+        <v>680</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>674</v>
+        <v>681</v>
       </c>
       <c r="E5" s="25" t="s">
         <v>72</v>
@@ -9754,13 +9774,13 @@
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="24" t="s">
-        <v>675</v>
+        <v>682</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>676</v>
+        <v>683</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>677</v>
+        <v>684</v>
       </c>
       <c r="E6" s="25" t="s">
         <v>72</v>
@@ -9768,27 +9788,27 @@
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="24" t="s">
-        <v>678</v>
+        <v>685</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>679</v>
+        <v>686</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
       <c r="E7" s="25" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="24" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="E8" s="25" t="s">
         <v>298</v>
@@ -9796,13 +9816,13 @@
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="24" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
       <c r="E9" s="25" t="s">
         <v>72</v>
@@ -9810,13 +9830,13 @@
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="24" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>689</v>
+        <v>696</v>
       </c>
       <c r="E10" s="25" t="s">
         <v>29</v>
@@ -9824,13 +9844,13 @@
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="24" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>692</v>
+        <v>699</v>
       </c>
       <c r="E11" s="25" t="s">
         <v>86</v>
@@ -9838,20 +9858,34 @@
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="24" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>695</v>
+        <v>702</v>
       </c>
       <c r="E12" s="25" t="s">
-        <v>86</v>
+        <v>298</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="24" t="s">
+        <v>703</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>704</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>705</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>298</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E5:E12">
+  <conditionalFormatting sqref="E5:E13">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Completed"</formula>
     </cfRule>
@@ -9866,7 +9900,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E12" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E13" type="list">
       <formula1>"Completed,In Progress,In Review,Planned"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9896,15 +9930,15 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="14" t="s">
-        <v>696</v>
+        <v>706</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="26" t="s">
-        <v>697</v>
+        <v>707</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9912,7 +9946,7 @@
         <v>29</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>699</v>
+        <v>709</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9920,7 +9954,7 @@
         <v>72</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9928,7 +9962,7 @@
         <v>298</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>701</v>
+        <v>711</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9936,7 +9970,7 @@
         <v>86</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>702</v>
+        <v>712</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9944,7 +9978,7 @@
         <v>21</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>703</v>
+        <v>713</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9952,15 +9986,15 @@
         <v>22</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="26" t="s">
-        <v>705</v>
+        <v>715</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>706</v>
+        <v>716</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9968,15 +10002,15 @@
         <v>20</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>707</v>
+        <v>717</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="26" t="s">
-        <v>708</v>
+        <v>718</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>709</v>
+        <v>719</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
For You to the Master: logged-out browsing, 24 per category, campaign cards, RB-33 pop-ups
- Feed, offer detail and categories open to logged-out shoppers (location
  via zip / lat+lng; empty until shared); feed capped at 24 per category
  and honors page_size
- Campaign cards: no campaign-level rating, N eligible products, Buy at;
  products carry their own rating + flavor / size
- Claim refusals add Master pop-up copy (title, message, note,
  days_remaining, starts_at, slot_limit); website shows all 10 pop-ups
- Email-code wording no longer promises a code was sent
- App handover updated (item 25)
</commit_message>
<xml_diff>
--- a/docs/client-requirements/Nibbl_Master_Requirements_Tracker.xlsx
+++ b/docs/client-requirements/Nibbl_Master_Requirements_Tracker.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1514" uniqueCount="727">
   <si>
     <t xml:space="preserve">Nibbl AI — Master Requirements Tracker</t>
   </si>
@@ -686,648 +686,648 @@
     <t xml:space="preserve">Campaign cards on For You (not product cards), category tabs, up to 24 per category</t>
   </si>
   <si>
-    <t xml:space="preserve">Campaign cards with category tabs.</t>
+    <t xml:space="preserve">For You: campaign cards only (brand, headline, description, reward badge, Going fast, Buy at, 'N eligible products · View Products'), no campaign-level rating (each product shows its own on the deal page), category tabs starting with For You, up to 24 per category in one vertical list. Logged-out shoppers browse after Allow Location / Enter ZIP (kept in their browser).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → Browse Offers Nearby / Offer tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open the site logged out, enter a ZIP, switch tabs, open a deal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile app: same API (documented).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retailer match = ranking boost; Any Retailer / Retailer Required verification (eligible / unclear → manual / ineligible)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upload receipts from different stores.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#10, #19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct entry: QR / Meta ad / URL bypasses geography only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campaign URL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open in a private window.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campaign-level suppression (never brand-wide)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claim one campaign of a brand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopper Rebate Flow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campaign details: products + ratings, Where to Buy, receipt eligibility, max rebate, offer eligibility, Going fast, share, save, Claim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offer page with all items.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopper Website</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → offer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open an offer; share and save.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#5, #10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserve Offer: prefill email/phone (collect if logged out), two required consents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserve Offer shows email + phone: prefilled when signed in (verified phone read-only), collected when logged out; both consents required. Logged-out shoppers open a deal from its link, then a 6-digit email code signs them in (or creates the account) before Confirm Reservation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → deal link → Continue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open a deal link logged out, enter email + phone, enter the code, Confirm &amp; Reserve.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile app: same API (documented for the app developer).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm Reservation screen: slot X of 5, exact deadline, Confirm &amp; Reserve (slot consumed only here)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot use shown on Reserve Offer; separate Confirm screen with product, retailer, reward, exact deadline and resulting slot use.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → offer → Continue → Confirm &amp; Reserve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claim an offer; check the deadline is 7 days out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservation eligibility checked before a claim slot is consumed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All checks (consent, slots, already claimed, cooldown, dates, capacity, funds) run before the slot is used.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Covered by automated tests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#17, #18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active claim slots (5) — occupied until approval, final rejection or expiry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → My Rewards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claim to the limit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Return Action Prompt: carousel, Submit Receipt + time left, Save for Later, My Offers badge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → home; header badge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claim, then return home.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rebate restriction pop-ups (10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All 10 Master pop-ups (RB-33) with Master titles, messages, notes and buttons: Consent required (Review &amp; Accept), All 5 claim slots in use / Already claimed (View My Offers), Please wait — N days remaining, One-time redeemed, Not started (date), Paused or ended, Today's rebates claimed (Explore + View My Offers), Receipt from an eligible retailer required (View Eligible Retailers), Offer no longer available. The API returns the copy (title, message, note, days_remaining, starts_at).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → deal → Continue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trigger consent, already-claimed and cooldown cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receipt Submission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submit inside the active campaign: requirements list, take/choose photo, review before submit, submitted state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-claim flow: Receipt Requirements (from the claim's locked terms), Take / Choose Photo, Review Your Receipt, Receipt submitted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → My Rewards → Upload receipt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upload a receipt for a claim.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receipt Validation &amp; Routing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capture date/time, retailer, transaction no., item, qty, net price, tax, total; clear date/retailer fail → reject; uncertain → manual; unreadable → new photo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upload clear / unclear / wrong-date receipts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OCR = AI service.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#19, #21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duplicate receipt + quantity allocation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upload the same receipt twice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receipt Outcomes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One resubmission before the original deadline (deadline never restarts)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First clear date/retailer rejection keeps the claim open with one resubmission; the second is final (claim closed, slot released). Purchase must be on or after the claim.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upload a receipt dated before the claim, then another.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outcome messages: accepted, manual review, unreadable, date, retailer, final rejection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master outcome screens: Purchase verified, Manual review, We couldn't read it, Date / Retailer does not qualify (with one resubmission), Final rejection.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → after submitting a receipt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trigger each outcome.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In-app + email decision notifications are tracked in Notifications &amp; Reminders.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notifications &amp; Reminders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receipt reminders 48h and 12h before the exact deadline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopper notifications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scheduled job sends both reminders.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservation confirmation, receipt submitted, approval/rejection (in-app + email), claim expiration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All five sent immediately in-app; approval and rejection also emailed (SES).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → notifications; email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claim, upload, get approved/rejected, let a claim expire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Push notification delivery (FCM / APNs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Push is a placeholder today.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting on client Firebase Workload Identity setup (EC2 role sent).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand Manual Review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">① Claim &amp; customer (email visible on every plan) · ② Full receipt viewer (zoom/rotate/download) · ③ Locked requirements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redemptions → Review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open a pending receipt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">④ Select line · ⑤ Confirm mapping + corrections (audit) · ⑥ Optional alias · ⑦ Calculated reward, rejection reasons, internal note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approve with alias; reject with reason.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand Redemptions Page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">① Summary (pending, approved, rejected, total paid) · ② Status tabs · ⑤ Priority queue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redemptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#21, #22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">③ Search &amp; filters (campaign, product, status, submitted date)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Search, campaign, product (via campaign products), status tabs, date range.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filter by campaign and product.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">⑥ Pagination &amp; Export CSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redemptions → Export CSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Export.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seven-day automatic approval (max reward, labelled, no alias, slot released)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check countdown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KPIs: total, pending 1–3★ response, average rating, review spend, cost per review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All five KPIs; spend from the wallet ledger.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviews → Review Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compare spend with the Wallet ledger.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabs (All, Published, 7-Day Hold, Flagged, Removed) + date range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabs with counts + date range + keyword search.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filters: rating, retailer, product, region</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All four (retailer from the receipt, region from the shopper's state).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filter by retailer and region.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review details: answers, final text, receipt evidence + gating summary, customer contact for service recovery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Side panel with answers, receipt, gating summary, masked email + copy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review Management → review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open a review.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#26, #33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low-rating response: countdown, Contact Customer, Add Brand Response, Flag for Removal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live countdown, Contact Customer (email), response, flag.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open a 2★ held review.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag reasons per Master (wrong product, unrelated, spam/fraud, PII, profanity, prohibited claim, other) + audit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master's 7 reasons, 500-char details, audit log.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review Management → Flag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag a review.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Export: Download CSV + Download Reviews; API integration Coming Soon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSV + readable reviews file, both with disclosure; API Coming Soon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review Management → Export</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Download both.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create Review Campaign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basics (required image), eligible products, controls, locked rules &amp; cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviews → Create</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a review campaign.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand question pool: add, suggest, Test Review Chat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Question pool: add, remove, ✨ Suggest Questions, and Test Review Chat (the same planned questions with answer chips and the AI draft; nothing saved or paid).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review Campaigns → Create / campaign page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run Test Review Chat to the draft.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Save Draft / Submit for Nibbl Review (published after review)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Save Draft / Submit for Nibbl Review; Admin → Campaign Approvals → Review campaigns tab: Approve / Request changes / Reject (comment required); brand sees status + Nibbl's comment and resubmits. Approved campaigns can be paused and resumed. Campaigns live before this release were grandfathered as approved.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review Campaigns; Admin → Campaign Approvals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submit a campaign, request changes in Admin, resubmit, approve.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live shopper preview (mobile)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live mobile preview of the shopper's review card (campaign image, Share your voice, $1 reward, 30 days left, Purchase verified, Claim $1) updates as the brand edits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change the image / products; the preview updates.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopper Review Opportunity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My Offers: Review Rewards card (Claim $1, Save for Later)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Review cards in the carousel and My Rewards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Get a receipt verified.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product Confirmed · Multiple Matches · Missing Consent · Share Your Voice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website: review card (Share your voice · $1 · days left · Claim $1) → Product Confirmed (or This isn't my product) → Multiple Matches when receipt wording fits several variants → Missing Consent only when missing → Share Your Voice → chat.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → My Offers → review card</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buy a product sold in two flavors under one name; pick the right one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobile app screens are the app developer's.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Developer rules: scan all lines, 0/1/many opportunities, cooldown per shopper+product, $1 reserve, no second verification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI Chat Review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product context loaded; rotating brand question; generated title &amp; review; edit; regenerate; final approval; $1 at any rating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → review chat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complete a review.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Five adaptive product questions with suggested answer chips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed AI questions today.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adaptive questions wait on the AI service endpoint; suggested-answer chips not built.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Separate 'recommend' and 'purchase again' questions; title 100 / body 500 limits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Separate recommend and buy-again questions with Yes, definitely / Maybe / No chips (answers saved as would-recommend / would-buy-again); title ≤ 100 and body ≤ 500 with counters, AI drafts trimmed to fit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complete a review; check the counters and chips.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratings &amp; Reviews Display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratings per product in campaign details; all reviews with sorting; review details + brand response; helpful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website → offer → reviews</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sort and mark helpful.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviews overview: rating, breakdown, % recommend, % would buy again, AI summary (positives + improvement)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rating, star breakdown, % recommend and % would buy again on the product reviews overview.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open an offer with reviews.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI summary (positives + improvement) waits on the AI service's summary endpoint; the backend hook is ready.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand Analytics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost &amp; Results · Customer &amp; Conversion · Campaign Performance (25-hour cycles)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analytics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compare cost with the ledger.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary, search &amp; filters, download opted-in, integrations Coming Soon, consent withdrawal rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filter and download.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table: brand activity, site activity, open claims, cooldowns, last active, status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columns per Master: Customer, Contact, Brand Activity (claims / rebates / reviews), Site Activity (total claims / % completion / reviews), Open Claims, Cooldowns (days left), Last Active, Status (Active / Banned), View. Tabs: All, Open Claim, Active Cooldown, Completed Rebate, Banned, Inactive.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open Customers; check each column and tab against a shopper with an open claim and a cooldown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Header (opt-in badges, status) + Ban Customer with reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Header: name, contact, customer since, last active, Nibbl Opt-In + brand Opt-In badges, Active/Banned. Ban modal with reason (suspicious activity, altered receipts, abuse, other); banned shoppers can't claim or get review opportunities from the brand; existing claims stay valid. Lift Ban.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers → View → Ban Customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ban with a reason; status shows Banned with the reason; Lift Ban restores it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relationship with brand · Nibbl activity totals · Recent activity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relationship tiles (claims, completed rebates, conversion, rewards, reviews, open claims); Nibbl totals only (claims, completion, reviews, rewards) — other brands' data never shown; recent activity timeline for this brand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers → View</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open a profile; totals match the shopper's history.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open claims · Cooldowns with Remove (confirmation + audit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open claims with days left. Rebate and review cooldowns with Remove → confirmation → cooldown cleared and an audit-log entry (who, when, which). Managers only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers → View → Cooldowns → Remove</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove a cooldown; the shopper can claim/review again; the audit log shows the removal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redemption history: full receipt 30 days, then matching line only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redemption history with View receipt + days left for 30 days; afterwards only the matching line item(s) are shown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers → View → Redemption History</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recent receipt shows View receipt; one older than 30 days shows Matching line only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand Wallet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balances: Available, Reserved, Promotional (definitions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wallet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check balances.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campaign Funding: 7-day need vs Available, funded status, reservations split</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wallet → Campaign Funding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activate a campaign.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automatic refill (Stripe): trigger 25%, fixed amount, recommendation, failure alert</t>
   </si>
   <si>
     <t xml:space="preserve">In Progress</t>
   </si>
   <si>
-    <t xml:space="preserve">Browse a category.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24-per-category cap and 'N eligible products' line to confirm.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retailer match = ranking boost; Any Retailer / Retailer Required verification (eligible / unclear → manual / ineligible)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upload receipts from different stores.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#10, #19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Direct entry: QR / Meta ad / URL bypasses geography only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campaign URL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open in a private window.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campaign-level suppression (never brand-wide)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claim one campaign of a brand.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shopper Rebate Flow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campaign details: products + ratings, Where to Buy, receipt eligibility, max rebate, offer eligibility, Going fast, share, save, Claim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offer page with all items.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shopper Website</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → offer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open an offer; share and save.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#5, #10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserve Offer: prefill email/phone (collect if logged out), two required consents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserve Offer shows email + phone: prefilled when signed in (verified phone read-only), collected when logged out; both consents required. Logged-out shoppers open a deal from its link, then a 6-digit email code signs them in (or creates the account) before Confirm Reservation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → deal link → Continue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open a deal link logged out, enter email + phone, enter the code, Confirm &amp; Reserve.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mobile app: same API (documented for the app developer).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm Reservation screen: slot X of 5, exact deadline, Confirm &amp; Reserve (slot consumed only here)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slot use shown on Reserve Offer; separate Confirm screen with product, retailer, reward, exact deadline and resulting slot use.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → offer → Continue → Confirm &amp; Reserve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claim an offer; check the deadline is 7 days out.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservation eligibility checked before a claim slot is consumed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All checks (consent, slots, already claimed, cooldown, dates, capacity, funds) run before the slot is used.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covered by automated tests.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#17, #18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Active claim slots (5) — occupied until approval, final rejection or expiry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → My Rewards</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claim to the limit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Return Action Prompt: carousel, Submit Receipt + time left, Save for Later, My Offers badge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → home; header badge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claim, then return home.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rebate restriction pop-ups (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All with own code; consent, slots, claimed, cooldown, one-time, not started, paused, capacity, funds; retailer shown on offer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → offer → Claim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trigger each case.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Align titles/buttons exactly with the Master pop-up mockup (e.g. 'Review &amp; Accept', 'N days remaining', 'View Eligible Retailers').</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Receipt Submission</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Submit inside the active campaign: requirements list, take/choose photo, review before submit, submitted state</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Per-claim flow: Receipt Requirements (from the claim's locked terms), Take / Choose Photo, Review Your Receipt, Receipt submitted.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → My Rewards → Upload receipt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upload a receipt for a claim.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Receipt Validation &amp; Routing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capture date/time, retailer, transaction no., item, qty, net price, tax, total; clear date/retailer fail → reject; uncertain → manual; unreadable → new photo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upload clear / unclear / wrong-date receipts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OCR = AI service.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#19, #21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Duplicate receipt + quantity allocation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upload the same receipt twice.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Receipt Outcomes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One resubmission before the original deadline (deadline never restarts)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First clear date/retailer rejection keeps the claim open with one resubmission; the second is final (claim closed, slot released). Purchase must be on or after the claim.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upload a receipt dated before the claim, then another.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outcome messages: accepted, manual review, unreadable, date, retailer, final rejection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Master outcome screens: Purchase verified, Manual review, We couldn't read it, Date / Retailer does not qualify (with one resubmission), Final rejection.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → after submitting a receipt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trigger each outcome.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In-app + email decision notifications are tracked in Notifications &amp; Reminders.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notifications &amp; Reminders</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Receipt reminders 48h and 12h before the exact deadline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shopper notifications</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scheduled job sends both reminders.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservation confirmation, receipt submitted, approval/rejection (in-app + email), claim expiration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All five sent immediately in-app; approval and rejection also emailed (SES).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → notifications; email</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claim, upload, get approved/rejected, let a claim expire.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Push notification delivery (FCM / APNs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Push is a placeholder today.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In Review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waiting on client Firebase Workload Identity setup (EC2 role sent).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand Manual Review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">① Claim &amp; customer (email visible on every plan) · ② Full receipt viewer (zoom/rotate/download) · ③ Locked requirements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redemptions → Review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open a pending receipt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">④ Select line · ⑤ Confirm mapping + corrections (audit) · ⑥ Optional alias · ⑦ Calculated reward, rejection reasons, internal note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approve with alias; reject with reason.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand Redemptions Page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">① Summary (pending, approved, rejected, total paid) · ② Status tabs · ⑤ Priority queue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redemptions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#21, #22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">③ Search &amp; filters (campaign, product, status, submitted date)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Search, campaign, product (via campaign products), status tabs, date range.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filter by campaign and product.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⑥ Pagination &amp; Export CSV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redemptions → Export CSV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Export.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seven-day automatic approval (max reward, labelled, no alias, slot released)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check countdown.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review Management</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KPIs: total, pending 1–3★ response, average rating, review spend, cost per review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All five KPIs; spend from the wallet ledger.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reviews → Review Management</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compare spend with the Wallet ledger.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tabs (All, Published, 7-Day Hold, Flagged, Removed) + date range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tabs with counts + date range + keyword search.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filters: rating, retailer, product, region</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All four (retailer from the receipt, region from the shopper's state).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filter by retailer and region.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review details: answers, final text, receipt evidence + gating summary, customer contact for service recovery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Side panel with answers, receipt, gating summary, masked email + copy.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review Management → review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open a review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#26, #33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low-rating response: countdown, Contact Customer, Add Brand Response, Flag for Removal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Live countdown, Contact Customer (email), response, flag.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open a 2★ held review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flag reasons per Master (wrong product, unrelated, spam/fraud, PII, profanity, prohibited claim, other) + audit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Master's 7 reasons, 500-char details, audit log.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review Management → Flag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flag a review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Export: Download CSV + Download Reviews; API integration Coming Soon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CSV + readable reviews file, both with disclosure; API Coming Soon.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review Management → Export</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Download both.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create Review Campaign</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Basics (required image), eligible products, controls, locked rules &amp; cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reviews → Create</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create a review campaign.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand question pool: add, suggest, Test Review Chat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Question pool: add, remove, ✨ Suggest Questions, and Test Review Chat (the same planned questions with answer chips and the AI draft; nothing saved or paid).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review Campaigns → Create / campaign page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run Test Review Chat to the draft.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Save Draft / Submit for Nibbl Review (published after review)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Save Draft / Submit for Nibbl Review; Admin → Campaign Approvals → Review campaigns tab: Approve / Request changes / Reject (comment required); brand sees status + Nibbl's comment and resubmits. Approved campaigns can be paused and resumed. Campaigns live before this release were grandfathered as approved.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review Campaigns; Admin → Campaign Approvals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Submit a campaign, request changes in Admin, resubmit, approve.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Live shopper preview (mobile)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Live mobile preview of the shopper's review card (campaign image, Share your voice, $1 reward, 30 days left, Purchase verified, Claim $1) updates as the brand edits.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Change the image / products; the preview updates.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shopper Review Opportunity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">My Offers: Review Rewards card (Claim $1, Save for Later)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review cards in the carousel and My Rewards.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Get a receipt verified.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Product Confirmed · Multiple Matches · Missing Consent · Share Your Voice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website: review card (Share your voice · $1 · days left · Claim $1) → Product Confirmed (or This isn't my product) → Multiple Matches when receipt wording fits several variants → Missing Consent only when missing → Share Your Voice → chat.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → My Offers → review card</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buy a product sold in two flavors under one name; pick the right one.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mobile app screens are the app developer's.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Developer rules: scan all lines, 0/1/many opportunities, cooldown per shopper+product, $1 reserve, no second verification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI Chat Review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Product context loaded; rotating brand question; generated title &amp; review; edit; regenerate; final approval; $1 at any rating</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → review chat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Complete a review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Five adaptive product questions with suggested answer chips</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fixed AI questions today.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adaptive questions wait on the AI service endpoint; suggested-answer chips not built.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Separate 'recommend' and 'purchase again' questions; title 100 / body 500 limits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Separate recommend and buy-again questions with Yes, definitely / Maybe / No chips (answers saved as would-recommend / would-buy-again); title ≤ 100 and body ≤ 500 with counters, AI drafts trimmed to fit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Complete a review; check the counters and chips.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ratings &amp; Reviews Display</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ratings per product in campaign details; all reviews with sorting; review details + brand response; helpful</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website → offer → reviews</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sort and mark helpful.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reviews overview: rating, breakdown, % recommend, % would buy again, AI summary (positives + improvement)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rating, star breakdown, % recommend and % would buy again on the product reviews overview.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open an offer with reviews.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI summary (positives + improvement) waits on the AI service's summary endpoint; the backend hook is ready.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand Analytics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cost &amp; Results · Customer &amp; Conversion · Campaign Performance (25-hour cycles)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analytics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compare cost with the ledger.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summary, search &amp; filters, download opted-in, integrations Coming Soon, consent withdrawal rule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filter and download.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table: brand activity, site activity, open claims, cooldowns, last active, status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Columns per Master: Customer, Contact, Brand Activity (claims / rebates / reviews), Site Activity (total claims / % completion / reviews), Open Claims, Cooldowns (days left), Last Active, Status (Active / Banned), View. Tabs: All, Open Claim, Active Cooldown, Completed Rebate, Banned, Inactive.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open Customers; check each column and tab against a shopper with an open claim and a cooldown.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customer Profile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Header (opt-in badges, status) + Ban Customer with reason</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Header: name, contact, customer since, last active, Nibbl Opt-In + brand Opt-In badges, Active/Banned. Ban modal with reason (suspicious activity, altered receipts, abuse, other); banned shoppers can't claim or get review opportunities from the brand; existing claims stay valid. Lift Ban.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customers → View → Ban Customer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ban with a reason; status shows Banned with the reason; Lift Ban restores it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relationship with brand · Nibbl activity totals · Recent activity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relationship tiles (claims, completed rebates, conversion, rewards, reviews, open claims); Nibbl totals only (claims, completion, reviews, rewards) — other brands' data never shown; recent activity timeline for this brand.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customers → View</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open a profile; totals match the shopper's history.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open claims · Cooldowns with Remove (confirmation + audit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open claims with days left. Rebate and review cooldowns with Remove → confirmation → cooldown cleared and an audit-log entry (who, when, which). Managers only.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customers → View → Cooldowns → Remove</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remove a cooldown; the shopper can claim/review again; the audit log shows the removal.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redemption history: full receipt 30 days, then matching line only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Redemption history with View receipt + days left for 30 days; afterwards only the matching line item(s) are shown.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Customers → View → Redemption History</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recent receipt shows View receipt; one older than 30 days shows Matching line only.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand Wallet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Balances: Available, Reserved, Promotional (definitions)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wallet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check balances.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campaign Funding: 7-day need vs Available, funded status, reservations split</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wallet → Campaign Funding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Activate a campaign.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Automatic refill (Stripe): trigger 25%, fixed amount, recommendation, failure alert</t>
-  </si>
-  <si>
     <t xml:space="preserve">Wallet → Auto-refill</t>
   </si>
   <si>
@@ -1725,9 +1725,6 @@
   </si>
   <si>
     <t xml:space="preserve">Sign in with a code; open My Offers, Wallet and Profile.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mobile app: same API (documented).</t>
   </si>
   <si>
     <t xml:space="preserve">Profile &amp; account security: verified phone locked; change via admin with re-verification; history</t>
@@ -3053,11 +3050,11 @@
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"Completed")</f>
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"In Progress")</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"In Review")</f>
@@ -3069,7 +3066,7 @@
       </c>
       <c r="H5" s="5" t="n">
         <f aca="false">IF(C5&gt;0,D5/C5,0)</f>
-        <v>0.946666666666667</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4595,7 +4592,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="132" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="9" t="n">
         <v>44</v>
       </c>
@@ -4609,7 +4606,7 @@
         <v>219</v>
       </c>
       <c r="F52" s="11" t="s">
-        <v>220</v>
+        <v>29</v>
       </c>
       <c r="G52" s="10" t="s">
         <v>205</v>
@@ -4618,7 +4615,7 @@
         <v>206</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="J52" s="10" t="s">
         <v>221</v>
@@ -4937,7 +4934,7 @@
       <c r="L61" s="12"/>
       <c r="M61" s="13"/>
     </row>
-    <row r="62" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="159.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="9" t="n">
         <v>54</v>
       </c>
@@ -4951,7 +4948,7 @@
         <v>261</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>220</v>
+        <v>29</v>
       </c>
       <c r="G62" s="10" t="s">
         <v>205</v>
@@ -4965,9 +4962,7 @@
       <c r="J62" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="K62" s="10" t="s">
-        <v>264</v>
-      </c>
+      <c r="K62" s="10"/>
       <c r="L62" s="12"/>
       <c r="M62" s="13" t="s">
         <v>253</v>
@@ -4978,13 +4973,13 @@
         <v>55</v>
       </c>
       <c r="C63" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="D63" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="D63" s="10" t="s">
+      <c r="E63" s="10" t="s">
         <v>266</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>267</v>
       </c>
       <c r="F63" s="11" t="s">
         <v>29</v>
@@ -4996,15 +4991,15 @@
         <v>206</v>
       </c>
       <c r="I63" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="J63" s="10" t="s">
         <v>268</v>
-      </c>
-      <c r="J63" s="10" t="s">
-        <v>269</v>
       </c>
       <c r="K63" s="10"/>
       <c r="L63" s="12"/>
       <c r="M63" s="13" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5012,10 +5007,10 @@
         <v>56</v>
       </c>
       <c r="C64" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="D64" s="10" t="s">
         <v>271</v>
-      </c>
-      <c r="D64" s="10" t="s">
-        <v>272</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>59</v>
@@ -5033,14 +5028,14 @@
         <v>172</v>
       </c>
       <c r="J64" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="K64" s="10" t="s">
         <v>273</v>
-      </c>
-      <c r="K64" s="10" t="s">
-        <v>274</v>
       </c>
       <c r="L64" s="12"/>
       <c r="M64" s="13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5048,10 +5043,10 @@
         <v>57</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>59</v>
@@ -5069,12 +5064,12 @@
         <v>172</v>
       </c>
       <c r="J65" s="10" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="K65" s="10"/>
       <c r="L65" s="12"/>
       <c r="M65" s="13" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5082,13 +5077,13 @@
         <v>58</v>
       </c>
       <c r="C66" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="D66" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="D66" s="10" t="s">
+      <c r="E66" s="10" t="s">
         <v>279</v>
-      </c>
-      <c r="E66" s="10" t="s">
-        <v>280</v>
       </c>
       <c r="F66" s="11" t="s">
         <v>29</v>
@@ -5100,15 +5095,15 @@
         <v>206</v>
       </c>
       <c r="I66" s="10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="J66" s="10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K66" s="10"/>
       <c r="L66" s="12"/>
       <c r="M66" s="13" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5116,13 +5111,13 @@
         <v>59</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D67" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="E67" s="10" t="s">
         <v>282</v>
-      </c>
-      <c r="E67" s="10" t="s">
-        <v>283</v>
       </c>
       <c r="F67" s="11" t="s">
         <v>29</v>
@@ -5134,17 +5129,17 @@
         <v>206</v>
       </c>
       <c r="I67" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="J67" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="J67" s="10" t="s">
+      <c r="K67" s="10" t="s">
         <v>285</v>
-      </c>
-      <c r="K67" s="10" t="s">
-        <v>286</v>
       </c>
       <c r="L67" s="12"/>
       <c r="M67" s="13" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5152,10 +5147,10 @@
         <v>60</v>
       </c>
       <c r="C68" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="D68" s="10" t="s">
         <v>287</v>
-      </c>
-      <c r="D68" s="10" t="s">
-        <v>288</v>
       </c>
       <c r="E68" s="10" t="s">
         <v>59</v>
@@ -5170,15 +5165,15 @@
         <v>206</v>
       </c>
       <c r="I68" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="J68" s="10" t="s">
         <v>289</v>
-      </c>
-      <c r="J68" s="10" t="s">
-        <v>290</v>
       </c>
       <c r="K68" s="10"/>
       <c r="L68" s="12"/>
       <c r="M68" s="13" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5186,13 +5181,13 @@
         <v>61</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D69" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="E69" s="10" t="s">
         <v>292</v>
-      </c>
-      <c r="E69" s="10" t="s">
-        <v>293</v>
       </c>
       <c r="F69" s="11" t="s">
         <v>29</v>
@@ -5204,15 +5199,15 @@
         <v>206</v>
       </c>
       <c r="I69" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="J69" s="10" t="s">
         <v>294</v>
-      </c>
-      <c r="J69" s="10" t="s">
-        <v>295</v>
       </c>
       <c r="K69" s="10"/>
       <c r="L69" s="12"/>
       <c r="M69" s="13" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5220,16 +5215,16 @@
         <v>62</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D70" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="E70" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="E70" s="10" t="s">
+      <c r="F70" s="11" t="s">
         <v>297</v>
-      </c>
-      <c r="F70" s="11" t="s">
-        <v>298</v>
       </c>
       <c r="G70" s="10" t="s">
         <v>171</v>
@@ -5244,7 +5239,7 @@
         <v>31</v>
       </c>
       <c r="K70" s="10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="L70" s="12"/>
       <c r="M70" s="13" t="s">
@@ -5256,10 +5251,10 @@
         <v>63</v>
       </c>
       <c r="C71" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="D71" s="10" t="s">
         <v>300</v>
-      </c>
-      <c r="D71" s="10" t="s">
-        <v>301</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>59</v>
@@ -5274,15 +5269,15 @@
         <v>31</v>
       </c>
       <c r="I71" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="J71" s="10" t="s">
         <v>302</v>
-      </c>
-      <c r="J71" s="10" t="s">
-        <v>303</v>
       </c>
       <c r="K71" s="10"/>
       <c r="L71" s="12"/>
       <c r="M71" s="13" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5290,10 +5285,10 @@
         <v>64</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E72" s="10" t="s">
         <v>59</v>
@@ -5308,15 +5303,15 @@
         <v>31</v>
       </c>
       <c r="I72" s="10" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J72" s="10" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="K72" s="10"/>
       <c r="L72" s="12"/>
       <c r="M72" s="13" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5324,10 +5319,10 @@
         <v>65</v>
       </c>
       <c r="C73" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="D73" s="10" t="s">
         <v>307</v>
-      </c>
-      <c r="D73" s="10" t="s">
-        <v>308</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>59</v>
@@ -5342,7 +5337,7 @@
         <v>31</v>
       </c>
       <c r="I73" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J73" s="10" t="s">
         <v>111</v>
@@ -5350,7 +5345,7 @@
       <c r="K73" s="10"/>
       <c r="L73" s="12"/>
       <c r="M73" s="13" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5358,13 +5353,13 @@
         <v>66</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D74" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="E74" s="10" t="s">
         <v>311</v>
-      </c>
-      <c r="E74" s="10" t="s">
-        <v>312</v>
       </c>
       <c r="F74" s="11" t="s">
         <v>29</v>
@@ -5376,15 +5371,15 @@
         <v>31</v>
       </c>
       <c r="I74" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J74" s="10" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="K74" s="10"/>
       <c r="L74" s="12"/>
       <c r="M74" s="13" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5392,10 +5387,10 @@
         <v>67</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>59</v>
@@ -5410,15 +5405,15 @@
         <v>31</v>
       </c>
       <c r="I75" s="10" t="s">
+        <v>314</v>
+      </c>
+      <c r="J75" s="10" t="s">
         <v>315</v>
-      </c>
-      <c r="J75" s="10" t="s">
-        <v>316</v>
       </c>
       <c r="K75" s="10"/>
       <c r="L75" s="12"/>
       <c r="M75" s="13" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5426,10 +5421,10 @@
         <v>68</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E76" s="10" t="s">
         <v>59</v>
@@ -5444,15 +5439,15 @@
         <v>31</v>
       </c>
       <c r="I76" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J76" s="10" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="K76" s="10"/>
       <c r="L76" s="12"/>
       <c r="M76" s="13" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5460,13 +5455,13 @@
         <v>69</v>
       </c>
       <c r="C77" s="10" t="s">
+        <v>319</v>
+      </c>
+      <c r="D77" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="D77" s="10" t="s">
+      <c r="E77" s="10" t="s">
         <v>321</v>
-      </c>
-      <c r="E77" s="10" t="s">
-        <v>322</v>
       </c>
       <c r="F77" s="11" t="s">
         <v>29</v>
@@ -5478,15 +5473,15 @@
         <v>31</v>
       </c>
       <c r="I77" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="J77" s="10" t="s">
         <v>323</v>
-      </c>
-      <c r="J77" s="10" t="s">
-        <v>324</v>
       </c>
       <c r="K77" s="10"/>
       <c r="L77" s="12"/>
       <c r="M77" s="13" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5494,13 +5489,13 @@
         <v>70</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D78" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="E78" s="10" t="s">
         <v>326</v>
-      </c>
-      <c r="E78" s="10" t="s">
-        <v>327</v>
       </c>
       <c r="F78" s="11" t="s">
         <v>29</v>
@@ -5512,7 +5507,7 @@
         <v>31</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J78" s="10" t="s">
         <v>111</v>
@@ -5520,7 +5515,7 @@
       <c r="K78" s="10"/>
       <c r="L78" s="12"/>
       <c r="M78" s="13" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5528,13 +5523,13 @@
         <v>71</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D79" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="E79" s="10" t="s">
         <v>328</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>329</v>
       </c>
       <c r="F79" s="11" t="s">
         <v>29</v>
@@ -5546,15 +5541,15 @@
         <v>31</v>
       </c>
       <c r="I79" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J79" s="10" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="K79" s="10"/>
       <c r="L79" s="12"/>
       <c r="M79" s="13" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5562,13 +5557,13 @@
         <v>72</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D80" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="E80" s="10" t="s">
         <v>331</v>
-      </c>
-      <c r="E80" s="10" t="s">
-        <v>332</v>
       </c>
       <c r="F80" s="11" t="s">
         <v>29</v>
@@ -5580,15 +5575,15 @@
         <v>31</v>
       </c>
       <c r="I80" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="J80" s="10" t="s">
         <v>333</v>
-      </c>
-      <c r="J80" s="10" t="s">
-        <v>334</v>
       </c>
       <c r="K80" s="10"/>
       <c r="L80" s="12"/>
       <c r="M80" s="13" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5596,13 +5591,13 @@
         <v>73</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D81" s="10" t="s">
+        <v>335</v>
+      </c>
+      <c r="E81" s="10" t="s">
         <v>336</v>
-      </c>
-      <c r="E81" s="10" t="s">
-        <v>337</v>
       </c>
       <c r="F81" s="11" t="s">
         <v>29</v>
@@ -5614,15 +5609,15 @@
         <v>31</v>
       </c>
       <c r="I81" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J81" s="10" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="K81" s="10"/>
       <c r="L81" s="12"/>
       <c r="M81" s="13" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5630,13 +5625,13 @@
         <v>74</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D82" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="E82" s="10" t="s">
         <v>339</v>
-      </c>
-      <c r="E82" s="10" t="s">
-        <v>340</v>
       </c>
       <c r="F82" s="11" t="s">
         <v>29</v>
@@ -5648,15 +5643,15 @@
         <v>31</v>
       </c>
       <c r="I82" s="10" t="s">
+        <v>340</v>
+      </c>
+      <c r="J82" s="10" t="s">
         <v>341</v>
-      </c>
-      <c r="J82" s="10" t="s">
-        <v>342</v>
       </c>
       <c r="K82" s="10"/>
       <c r="L82" s="12"/>
       <c r="M82" s="13" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5664,13 +5659,13 @@
         <v>75</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D83" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="E83" s="10" t="s">
         <v>343</v>
-      </c>
-      <c r="E83" s="10" t="s">
-        <v>344</v>
       </c>
       <c r="F83" s="11" t="s">
         <v>29</v>
@@ -5682,15 +5677,15 @@
         <v>31</v>
       </c>
       <c r="I83" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="J83" s="10" t="s">
         <v>345</v>
-      </c>
-      <c r="J83" s="10" t="s">
-        <v>346</v>
       </c>
       <c r="K83" s="10"/>
       <c r="L83" s="12"/>
       <c r="M83" s="13" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5698,10 +5693,10 @@
         <v>76</v>
       </c>
       <c r="C84" s="10" t="s">
+        <v>346</v>
+      </c>
+      <c r="D84" s="10" t="s">
         <v>347</v>
-      </c>
-      <c r="D84" s="10" t="s">
-        <v>348</v>
       </c>
       <c r="E84" s="10" t="s">
         <v>59</v>
@@ -5716,15 +5711,15 @@
         <v>31</v>
       </c>
       <c r="I84" s="10" t="s">
+        <v>348</v>
+      </c>
+      <c r="J84" s="10" t="s">
         <v>349</v>
-      </c>
-      <c r="J84" s="10" t="s">
-        <v>350</v>
       </c>
       <c r="K84" s="10"/>
       <c r="L84" s="12"/>
       <c r="M84" s="13" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5732,13 +5727,13 @@
         <v>77</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D85" s="10" t="s">
+        <v>351</v>
+      </c>
+      <c r="E85" s="10" t="s">
         <v>352</v>
-      </c>
-      <c r="E85" s="10" t="s">
-        <v>353</v>
       </c>
       <c r="F85" s="11" t="s">
         <v>29</v>
@@ -5750,15 +5745,15 @@
         <v>31</v>
       </c>
       <c r="I85" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="J85" s="10" t="s">
         <v>354</v>
-      </c>
-      <c r="J85" s="10" t="s">
-        <v>355</v>
       </c>
       <c r="K85" s="10"/>
       <c r="L85" s="12"/>
       <c r="M85" s="13" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5766,13 +5761,13 @@
         <v>78</v>
       </c>
       <c r="C86" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D86" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="E86" s="10" t="s">
         <v>356</v>
-      </c>
-      <c r="E86" s="10" t="s">
-        <v>357</v>
       </c>
       <c r="F86" s="11" t="s">
         <v>29</v>
@@ -5784,15 +5779,15 @@
         <v>31</v>
       </c>
       <c r="I86" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="J86" s="10" t="s">
         <v>358</v>
-      </c>
-      <c r="J86" s="10" t="s">
-        <v>359</v>
       </c>
       <c r="K86" s="10"/>
       <c r="L86" s="12"/>
       <c r="M86" s="13" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5800,13 +5795,13 @@
         <v>79</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D87" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="E87" s="10" t="s">
         <v>360</v>
-      </c>
-      <c r="E87" s="10" t="s">
-        <v>361</v>
       </c>
       <c r="F87" s="11" t="s">
         <v>29</v>
@@ -5818,15 +5813,15 @@
         <v>31</v>
       </c>
       <c r="I87" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="J87" s="10" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="K87" s="10"/>
       <c r="L87" s="12"/>
       <c r="M87" s="13" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5834,13 +5829,13 @@
         <v>80</v>
       </c>
       <c r="C88" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="D88" s="10" t="s">
         <v>363</v>
       </c>
-      <c r="D88" s="10" t="s">
+      <c r="E88" s="10" t="s">
         <v>364</v>
-      </c>
-      <c r="E88" s="10" t="s">
-        <v>365</v>
       </c>
       <c r="F88" s="11" t="s">
         <v>29</v>
@@ -5855,12 +5850,12 @@
         <v>255</v>
       </c>
       <c r="J88" s="10" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="K88" s="10"/>
       <c r="L88" s="12"/>
       <c r="M88" s="13" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5868,13 +5863,13 @@
         <v>81</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D89" s="10" t="s">
+        <v>366</v>
+      </c>
+      <c r="E89" s="10" t="s">
         <v>367</v>
-      </c>
-      <c r="E89" s="10" t="s">
-        <v>368</v>
       </c>
       <c r="F89" s="11" t="s">
         <v>29</v>
@@ -5886,17 +5881,17 @@
         <v>206</v>
       </c>
       <c r="I89" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="J89" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J89" s="10" t="s">
+      <c r="K89" s="10" t="s">
         <v>370</v>
-      </c>
-      <c r="K89" s="10" t="s">
-        <v>371</v>
       </c>
       <c r="L89" s="12"/>
       <c r="M89" s="13" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5904,10 +5899,10 @@
         <v>82</v>
       </c>
       <c r="C90" s="10" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E90" s="10" t="s">
         <v>59</v>
@@ -5930,7 +5925,7 @@
       <c r="K90" s="10"/>
       <c r="L90" s="12"/>
       <c r="M90" s="13" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5938,10 +5933,10 @@
         <v>83</v>
       </c>
       <c r="C91" s="10" t="s">
+        <v>373</v>
+      </c>
+      <c r="D91" s="10" t="s">
         <v>374</v>
-      </c>
-      <c r="D91" s="10" t="s">
-        <v>375</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>59</v>
@@ -5956,15 +5951,15 @@
         <v>206</v>
       </c>
       <c r="I91" s="10" t="s">
+        <v>375</v>
+      </c>
+      <c r="J91" s="10" t="s">
         <v>376</v>
-      </c>
-      <c r="J91" s="10" t="s">
-        <v>377</v>
       </c>
       <c r="K91" s="10"/>
       <c r="L91" s="12"/>
       <c r="M91" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5972,16 +5967,16 @@
         <v>84</v>
       </c>
       <c r="C92" s="10" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D92" s="10" t="s">
+        <v>378</v>
+      </c>
+      <c r="E92" s="10" t="s">
         <v>379</v>
       </c>
-      <c r="E92" s="10" t="s">
-        <v>380</v>
-      </c>
       <c r="F92" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G92" s="10" t="s">
         <v>171</v>
@@ -5996,11 +5991,11 @@
         <v>31</v>
       </c>
       <c r="K92" s="10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="L92" s="12"/>
       <c r="M92" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6008,13 +6003,13 @@
         <v>85</v>
       </c>
       <c r="C93" s="10" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D93" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="E93" s="10" t="s">
         <v>382</v>
-      </c>
-      <c r="E93" s="10" t="s">
-        <v>383</v>
       </c>
       <c r="F93" s="11" t="s">
         <v>29</v>
@@ -6026,15 +6021,15 @@
         <v>206</v>
       </c>
       <c r="I93" s="10" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="J93" s="10" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="K93" s="10"/>
       <c r="L93" s="12"/>
       <c r="M93" s="13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6042,10 +6037,10 @@
         <v>86</v>
       </c>
       <c r="C94" s="10" t="s">
+        <v>384</v>
+      </c>
+      <c r="D94" s="10" t="s">
         <v>385</v>
-      </c>
-      <c r="D94" s="10" t="s">
-        <v>386</v>
       </c>
       <c r="E94" s="10" t="s">
         <v>59</v>
@@ -6060,15 +6055,15 @@
         <v>206</v>
       </c>
       <c r="I94" s="10" t="s">
+        <v>386</v>
+      </c>
+      <c r="J94" s="10" t="s">
         <v>387</v>
-      </c>
-      <c r="J94" s="10" t="s">
-        <v>388</v>
       </c>
       <c r="K94" s="10"/>
       <c r="L94" s="12"/>
       <c r="M94" s="13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6076,16 +6071,16 @@
         <v>87</v>
       </c>
       <c r="C95" s="10" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D95" s="10" t="s">
+        <v>389</v>
+      </c>
+      <c r="E95" s="10" t="s">
         <v>390</v>
       </c>
-      <c r="E95" s="10" t="s">
-        <v>391</v>
-      </c>
       <c r="F95" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G95" s="10" t="s">
         <v>205</v>
@@ -6094,17 +6089,17 @@
         <v>206</v>
       </c>
       <c r="I95" s="10" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="J95" s="10" t="s">
+        <v>391</v>
+      </c>
+      <c r="K95" s="10" t="s">
         <v>392</v>
-      </c>
-      <c r="K95" s="10" t="s">
-        <v>393</v>
       </c>
       <c r="L95" s="12"/>
       <c r="M95" s="13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6112,10 +6107,10 @@
         <v>88</v>
       </c>
       <c r="C96" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="D96" s="10" t="s">
         <v>394</v>
-      </c>
-      <c r="D96" s="10" t="s">
-        <v>395</v>
       </c>
       <c r="E96" s="10" t="s">
         <v>59</v>
@@ -6130,15 +6125,15 @@
         <v>31</v>
       </c>
       <c r="I96" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="J96" s="10" t="s">
         <v>396</v>
-      </c>
-      <c r="J96" s="10" t="s">
-        <v>397</v>
       </c>
       <c r="K96" s="10"/>
       <c r="L96" s="12"/>
       <c r="M96" s="13" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6146,10 +6141,10 @@
         <v>89</v>
       </c>
       <c r="C97" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="D97" s="10" t="s">
         <v>399</v>
-      </c>
-      <c r="D97" s="10" t="s">
-        <v>400</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>59</v>
@@ -6164,15 +6159,15 @@
         <v>31</v>
       </c>
       <c r="I97" s="10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="J97" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="K97" s="10"/>
       <c r="L97" s="12"/>
       <c r="M97" s="13" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6180,13 +6175,13 @@
         <v>90</v>
       </c>
       <c r="C98" s="10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D98" s="10" t="s">
+        <v>402</v>
+      </c>
+      <c r="E98" s="10" t="s">
         <v>403</v>
-      </c>
-      <c r="E98" s="10" t="s">
-        <v>404</v>
       </c>
       <c r="F98" s="11" t="s">
         <v>29</v>
@@ -6198,15 +6193,15 @@
         <v>31</v>
       </c>
       <c r="I98" s="10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="J98" s="10" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="K98" s="10"/>
       <c r="L98" s="12"/>
       <c r="M98" s="13" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6214,13 +6209,13 @@
         <v>91</v>
       </c>
       <c r="C99" s="10" t="s">
+        <v>405</v>
+      </c>
+      <c r="D99" s="10" t="s">
         <v>406</v>
       </c>
-      <c r="D99" s="10" t="s">
+      <c r="E99" s="10" t="s">
         <v>407</v>
-      </c>
-      <c r="E99" s="10" t="s">
-        <v>408</v>
       </c>
       <c r="F99" s="11" t="s">
         <v>29</v>
@@ -6232,15 +6227,15 @@
         <v>31</v>
       </c>
       <c r="I99" s="10" t="s">
+        <v>408</v>
+      </c>
+      <c r="J99" s="10" t="s">
         <v>409</v>
-      </c>
-      <c r="J99" s="10" t="s">
-        <v>410</v>
       </c>
       <c r="K99" s="10"/>
       <c r="L99" s="12"/>
       <c r="M99" s="13" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6248,13 +6243,13 @@
         <v>92</v>
       </c>
       <c r="C100" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D100" s="10" t="s">
+        <v>411</v>
+      </c>
+      <c r="E100" s="10" t="s">
         <v>412</v>
-      </c>
-      <c r="E100" s="10" t="s">
-        <v>413</v>
       </c>
       <c r="F100" s="11" t="s">
         <v>29</v>
@@ -6266,15 +6261,15 @@
         <v>31</v>
       </c>
       <c r="I100" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="J100" s="10" t="s">
         <v>414</v>
-      </c>
-      <c r="J100" s="10" t="s">
-        <v>415</v>
       </c>
       <c r="K100" s="10"/>
       <c r="L100" s="12"/>
       <c r="M100" s="13" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6282,13 +6277,13 @@
         <v>93</v>
       </c>
       <c r="C101" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D101" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="E101" s="10" t="s">
         <v>416</v>
-      </c>
-      <c r="E101" s="10" t="s">
-        <v>417</v>
       </c>
       <c r="F101" s="11" t="s">
         <v>29</v>
@@ -6300,15 +6295,15 @@
         <v>31</v>
       </c>
       <c r="I101" s="10" t="s">
+        <v>417</v>
+      </c>
+      <c r="J101" s="10" t="s">
         <v>418</v>
-      </c>
-      <c r="J101" s="10" t="s">
-        <v>419</v>
       </c>
       <c r="K101" s="10"/>
       <c r="L101" s="12"/>
       <c r="M101" s="13" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6316,13 +6311,13 @@
         <v>94</v>
       </c>
       <c r="C102" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D102" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="E102" s="10" t="s">
         <v>420</v>
-      </c>
-      <c r="E102" s="10" t="s">
-        <v>421</v>
       </c>
       <c r="F102" s="11" t="s">
         <v>29</v>
@@ -6334,15 +6329,15 @@
         <v>31</v>
       </c>
       <c r="I102" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="J102" s="10" t="s">
         <v>422</v>
-      </c>
-      <c r="J102" s="10" t="s">
-        <v>423</v>
       </c>
       <c r="K102" s="10"/>
       <c r="L102" s="12"/>
       <c r="M102" s="13" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6350,10 +6345,10 @@
         <v>95</v>
       </c>
       <c r="C103" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="D103" s="10" t="s">
         <v>424</v>
-      </c>
-      <c r="D103" s="10" t="s">
-        <v>425</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>59</v>
@@ -6368,15 +6363,15 @@
         <v>31</v>
       </c>
       <c r="I103" s="10" t="s">
+        <v>425</v>
+      </c>
+      <c r="J103" s="10" t="s">
         <v>426</v>
-      </c>
-      <c r="J103" s="10" t="s">
-        <v>427</v>
       </c>
       <c r="K103" s="10"/>
       <c r="L103" s="12"/>
       <c r="M103" s="13" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6384,10 +6379,10 @@
         <v>96</v>
       </c>
       <c r="C104" s="10" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D104" s="10" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="E104" s="10" t="s">
         <v>59</v>
@@ -6402,15 +6397,15 @@
         <v>31</v>
       </c>
       <c r="I104" s="10" t="s">
+        <v>429</v>
+      </c>
+      <c r="J104" s="10" t="s">
         <v>430</v>
-      </c>
-      <c r="J104" s="10" t="s">
-        <v>431</v>
       </c>
       <c r="K104" s="10"/>
       <c r="L104" s="12"/>
       <c r="M104" s="13" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6418,16 +6413,16 @@
         <v>97</v>
       </c>
       <c r="C105" s="10" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D105" s="10" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F105" s="11" t="s">
-        <v>220</v>
+        <v>432</v>
       </c>
       <c r="G105" s="10" t="s">
         <v>51</v>
@@ -6454,7 +6449,7 @@
         <v>98</v>
       </c>
       <c r="C106" s="10" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D106" s="10" t="s">
         <v>437</v>
@@ -6472,7 +6467,7 @@
         <v>31</v>
       </c>
       <c r="I106" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="J106" s="10" t="s">
         <v>438</v>
@@ -6488,7 +6483,7 @@
         <v>99</v>
       </c>
       <c r="C107" s="10" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D107" s="10" t="s">
         <v>440</v>
@@ -6703,7 +6698,7 @@
         <v>467</v>
       </c>
       <c r="F113" s="11" t="s">
-        <v>220</v>
+        <v>432</v>
       </c>
       <c r="G113" s="10" t="s">
         <v>51</v>
@@ -7129,7 +7124,7 @@
         <v>517</v>
       </c>
       <c r="J125" s="10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="K125" s="10"/>
       <c r="L125" s="12"/>
@@ -7253,7 +7248,7 @@
         <v>531</v>
       </c>
       <c r="F129" s="11" t="s">
-        <v>220</v>
+        <v>432</v>
       </c>
       <c r="G129" s="10" t="s">
         <v>205</v>
@@ -7508,7 +7503,7 @@
         <v>565</v>
       </c>
       <c r="K136" s="10" t="s">
-        <v>566</v>
+        <v>222</v>
       </c>
       <c r="L136" s="12"/>
       <c r="M136" s="13" t="s">
@@ -7523,10 +7518,10 @@
         <v>561</v>
       </c>
       <c r="D137" s="10" t="s">
+        <v>566</v>
+      </c>
+      <c r="E137" s="10" t="s">
         <v>567</v>
-      </c>
-      <c r="E137" s="10" t="s">
-        <v>568</v>
       </c>
       <c r="F137" s="11" t="s">
         <v>29</v>
@@ -7538,10 +7533,10 @@
         <v>206</v>
       </c>
       <c r="I137" s="10" t="s">
+        <v>568</v>
+      </c>
+      <c r="J137" s="10" t="s">
         <v>569</v>
-      </c>
-      <c r="J137" s="10" t="s">
-        <v>570</v>
       </c>
       <c r="K137" s="10"/>
       <c r="L137" s="12"/>
@@ -7554,35 +7549,35 @@
         <v>130</v>
       </c>
       <c r="C138" s="10" t="s">
+        <v>570</v>
+      </c>
+      <c r="D138" s="10" t="s">
         <v>571</v>
       </c>
-      <c r="D138" s="10" t="s">
+      <c r="E138" s="10" t="s">
         <v>572</v>
       </c>
-      <c r="E138" s="10" t="s">
+      <c r="F138" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G138" s="10" t="s">
         <v>573</v>
       </c>
-      <c r="F138" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G138" s="10" t="s">
+      <c r="H138" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I138" s="10" t="s">
         <v>574</v>
       </c>
-      <c r="H138" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I138" s="10" t="s">
+      <c r="J138" s="10" t="s">
         <v>575</v>
       </c>
-      <c r="J138" s="10" t="s">
+      <c r="K138" s="10" t="s">
         <v>576</v>
-      </c>
-      <c r="K138" s="10" t="s">
-        <v>577</v>
       </c>
       <c r="L138" s="12"/>
       <c r="M138" s="13" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7590,13 +7585,13 @@
         <v>131</v>
       </c>
       <c r="C139" s="10" t="s">
+        <v>578</v>
+      </c>
+      <c r="D139" s="10" t="s">
         <v>579</v>
       </c>
-      <c r="D139" s="10" t="s">
+      <c r="E139" s="10" t="s">
         <v>580</v>
-      </c>
-      <c r="E139" s="10" t="s">
-        <v>581</v>
       </c>
       <c r="F139" s="11" t="s">
         <v>29</v>
@@ -7608,13 +7603,13 @@
         <v>31</v>
       </c>
       <c r="I139" s="10" t="s">
+        <v>581</v>
+      </c>
+      <c r="J139" s="10" t="s">
         <v>582</v>
       </c>
-      <c r="J139" s="10" t="s">
+      <c r="K139" s="10" t="s">
         <v>583</v>
-      </c>
-      <c r="K139" s="10" t="s">
-        <v>584</v>
       </c>
       <c r="L139" s="12"/>
       <c r="M139" s="13" t="s">
@@ -7626,13 +7621,13 @@
         <v>132</v>
       </c>
       <c r="C140" s="10" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D140" s="10" t="s">
+        <v>584</v>
+      </c>
+      <c r="E140" s="10" t="s">
         <v>585</v>
-      </c>
-      <c r="E140" s="10" t="s">
-        <v>586</v>
       </c>
       <c r="F140" s="11" t="s">
         <v>29</v>
@@ -7644,13 +7639,13 @@
         <v>31</v>
       </c>
       <c r="I140" s="10" t="s">
+        <v>586</v>
+      </c>
+      <c r="J140" s="10" t="s">
         <v>587</v>
       </c>
-      <c r="J140" s="10" t="s">
+      <c r="K140" s="10" t="s">
         <v>588</v>
-      </c>
-      <c r="K140" s="10" t="s">
-        <v>589</v>
       </c>
       <c r="L140" s="12"/>
       <c r="M140" s="13" t="s">
@@ -7662,13 +7657,13 @@
         <v>133</v>
       </c>
       <c r="C141" s="10" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D141" s="10" t="s">
+        <v>589</v>
+      </c>
+      <c r="E141" s="10" t="s">
         <v>590</v>
-      </c>
-      <c r="E141" s="10" t="s">
-        <v>591</v>
       </c>
       <c r="F141" s="11" t="s">
         <v>29</v>
@@ -7680,10 +7675,10 @@
         <v>31</v>
       </c>
       <c r="I141" s="10" t="s">
+        <v>591</v>
+      </c>
+      <c r="J141" s="10" t="s">
         <v>592</v>
-      </c>
-      <c r="J141" s="10" t="s">
-        <v>593</v>
       </c>
       <c r="K141" s="10"/>
       <c r="L141" s="12"/>
@@ -7696,13 +7691,13 @@
         <v>134</v>
       </c>
       <c r="C142" s="10" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D142" s="10" t="s">
+        <v>593</v>
+      </c>
+      <c r="E142" s="10" t="s">
         <v>594</v>
-      </c>
-      <c r="E142" s="10" t="s">
-        <v>595</v>
       </c>
       <c r="F142" s="11" t="s">
         <v>29</v>
@@ -7714,15 +7709,15 @@
         <v>31</v>
       </c>
       <c r="I142" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="J142" s="10" t="s">
         <v>596</v>
-      </c>
-      <c r="J142" s="10" t="s">
-        <v>597</v>
       </c>
       <c r="K142" s="10"/>
       <c r="L142" s="12"/>
       <c r="M142" s="13" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7730,33 +7725,33 @@
         <v>135</v>
       </c>
       <c r="C143" s="10" t="s">
+        <v>598</v>
+      </c>
+      <c r="D143" s="10" t="s">
         <v>599</v>
       </c>
-      <c r="D143" s="10" t="s">
+      <c r="E143" s="10" t="s">
         <v>600</v>
       </c>
-      <c r="E143" s="10" t="s">
+      <c r="F143" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G143" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="H143" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I143" s="10" t="s">
         <v>601</v>
       </c>
-      <c r="F143" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G143" s="10" t="s">
-        <v>574</v>
-      </c>
-      <c r="H143" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I143" s="10" t="s">
+      <c r="J143" s="10" t="s">
         <v>602</v>
-      </c>
-      <c r="J143" s="10" t="s">
-        <v>603</v>
       </c>
       <c r="K143" s="10"/>
       <c r="L143" s="12"/>
       <c r="M143" s="13" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7764,33 +7759,33 @@
         <v>136</v>
       </c>
       <c r="C144" s="10" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="D144" s="10" t="s">
+        <v>604</v>
+      </c>
+      <c r="E144" s="10" t="s">
         <v>605</v>
       </c>
-      <c r="E144" s="10" t="s">
+      <c r="F144" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G144" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="H144" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I144" s="10" t="s">
         <v>606</v>
       </c>
-      <c r="F144" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G144" s="10" t="s">
-        <v>574</v>
-      </c>
-      <c r="H144" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I144" s="10" t="s">
+      <c r="J144" s="10" t="s">
         <v>607</v>
-      </c>
-      <c r="J144" s="10" t="s">
-        <v>608</v>
       </c>
       <c r="K144" s="10"/>
       <c r="L144" s="12"/>
       <c r="M144" s="13" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7798,10 +7793,10 @@
         <v>137</v>
       </c>
       <c r="C145" s="10" t="s">
+        <v>609</v>
+      </c>
+      <c r="D145" s="10" t="s">
         <v>610</v>
-      </c>
-      <c r="D145" s="10" t="s">
-        <v>611</v>
       </c>
       <c r="E145" s="10" t="s">
         <v>59</v>
@@ -7810,21 +7805,21 @@
         <v>29</v>
       </c>
       <c r="G145" s="10" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="H145" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I145" s="10" t="s">
+        <v>611</v>
+      </c>
+      <c r="J145" s="10" t="s">
         <v>612</v>
-      </c>
-      <c r="J145" s="10" t="s">
-        <v>613</v>
       </c>
       <c r="K145" s="10"/>
       <c r="L145" s="12"/>
       <c r="M145" s="13" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7832,10 +7827,10 @@
         <v>138</v>
       </c>
       <c r="C146" s="10" t="s">
+        <v>614</v>
+      </c>
+      <c r="D146" s="10" t="s">
         <v>615</v>
-      </c>
-      <c r="D146" s="10" t="s">
-        <v>616</v>
       </c>
       <c r="E146" s="10" t="s">
         <v>59</v>
@@ -7844,21 +7839,21 @@
         <v>29</v>
       </c>
       <c r="G146" s="10" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="H146" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I146" s="10" t="s">
+        <v>616</v>
+      </c>
+      <c r="J146" s="10" t="s">
         <v>617</v>
-      </c>
-      <c r="J146" s="10" t="s">
-        <v>618</v>
       </c>
       <c r="K146" s="10"/>
       <c r="L146" s="12"/>
       <c r="M146" s="13" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7866,33 +7861,33 @@
         <v>139</v>
       </c>
       <c r="C147" s="10" t="s">
+        <v>618</v>
+      </c>
+      <c r="D147" s="10" t="s">
         <v>619</v>
       </c>
-      <c r="D147" s="10" t="s">
+      <c r="E147" s="10" t="s">
         <v>620</v>
       </c>
-      <c r="E147" s="10" t="s">
+      <c r="F147" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G147" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="H147" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I147" s="10" t="s">
         <v>621</v>
       </c>
-      <c r="F147" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G147" s="10" t="s">
-        <v>574</v>
-      </c>
-      <c r="H147" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I147" s="10" t="s">
+      <c r="J147" s="10" t="s">
         <v>622</v>
-      </c>
-      <c r="J147" s="10" t="s">
-        <v>623</v>
       </c>
       <c r="K147" s="10"/>
       <c r="L147" s="12"/>
       <c r="M147" s="13" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="132" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7900,33 +7895,33 @@
         <v>140</v>
       </c>
       <c r="C148" s="10" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D148" s="10" t="s">
+        <v>623</v>
+      </c>
+      <c r="E148" s="10" t="s">
         <v>624</v>
       </c>
-      <c r="E148" s="10" t="s">
+      <c r="F148" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G148" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="H148" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I148" s="10" t="s">
         <v>625</v>
       </c>
-      <c r="F148" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G148" s="10" t="s">
-        <v>574</v>
-      </c>
-      <c r="H148" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I148" s="10" t="s">
+      <c r="J148" s="10" t="s">
         <v>626</v>
-      </c>
-      <c r="J148" s="10" t="s">
-        <v>627</v>
       </c>
       <c r="K148" s="10"/>
       <c r="L148" s="12"/>
       <c r="M148" s="13" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7934,33 +7929,33 @@
         <v>141</v>
       </c>
       <c r="C149" s="10" t="s">
+        <v>628</v>
+      </c>
+      <c r="D149" s="10" t="s">
         <v>629</v>
       </c>
-      <c r="D149" s="10" t="s">
+      <c r="E149" s="10" t="s">
         <v>630</v>
       </c>
-      <c r="E149" s="10" t="s">
+      <c r="F149" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G149" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="H149" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I149" s="10" t="s">
         <v>631</v>
       </c>
-      <c r="F149" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G149" s="10" t="s">
-        <v>574</v>
-      </c>
-      <c r="H149" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I149" s="10" t="s">
+      <c r="J149" s="10" t="s">
         <v>632</v>
-      </c>
-      <c r="J149" s="10" t="s">
-        <v>633</v>
       </c>
       <c r="K149" s="10"/>
       <c r="L149" s="12"/>
       <c r="M149" s="13" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7968,10 +7963,10 @@
         <v>142</v>
       </c>
       <c r="C150" s="10" t="s">
+        <v>633</v>
+      </c>
+      <c r="D150" s="10" t="s">
         <v>634</v>
-      </c>
-      <c r="D150" s="10" t="s">
-        <v>635</v>
       </c>
       <c r="E150" s="10" t="s">
         <v>59</v>
@@ -7980,21 +7975,21 @@
         <v>29</v>
       </c>
       <c r="G150" s="10" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="H150" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I150" s="10" t="s">
+        <v>635</v>
+      </c>
+      <c r="J150" s="10" t="s">
         <v>636</v>
-      </c>
-      <c r="J150" s="10" t="s">
-        <v>637</v>
       </c>
       <c r="K150" s="10"/>
       <c r="L150" s="12"/>
       <c r="M150" s="13" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8002,35 +7997,35 @@
         <v>143</v>
       </c>
       <c r="C151" s="10" t="s">
+        <v>638</v>
+      </c>
+      <c r="D151" s="10" t="s">
         <v>639</v>
       </c>
-      <c r="D151" s="10" t="s">
+      <c r="E151" s="10" t="s">
         <v>640</v>
       </c>
-      <c r="E151" s="10" t="s">
+      <c r="F151" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G151" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="H151" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I151" s="10" t="s">
         <v>641</v>
       </c>
-      <c r="F151" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G151" s="10" t="s">
-        <v>574</v>
-      </c>
-      <c r="H151" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I151" s="10" t="s">
+      <c r="J151" s="10" t="s">
         <v>642</v>
       </c>
-      <c r="J151" s="10" t="s">
+      <c r="K151" s="10" t="s">
         <v>643</v>
-      </c>
-      <c r="K151" s="10" t="s">
-        <v>644</v>
       </c>
       <c r="L151" s="12"/>
       <c r="M151" s="13" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8038,10 +8033,10 @@
         <v>144</v>
       </c>
       <c r="C152" s="10" t="s">
+        <v>645</v>
+      </c>
+      <c r="D152" s="10" t="s">
         <v>646</v>
-      </c>
-      <c r="D152" s="10" t="s">
-        <v>647</v>
       </c>
       <c r="E152" s="10" t="s">
         <v>59</v>
@@ -8050,23 +8045,23 @@
         <v>29</v>
       </c>
       <c r="G152" s="10" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="H152" s="10" t="s">
         <v>31</v>
       </c>
       <c r="I152" s="10" t="s">
+        <v>647</v>
+      </c>
+      <c r="J152" s="10" t="s">
         <v>648</v>
       </c>
-      <c r="J152" s="10" t="s">
+      <c r="K152" s="10" t="s">
         <v>649</v>
-      </c>
-      <c r="K152" s="10" t="s">
-        <v>650</v>
       </c>
       <c r="L152" s="12"/>
       <c r="M152" s="13" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8074,10 +8069,10 @@
         <v>145</v>
       </c>
       <c r="C153" s="10" t="s">
+        <v>651</v>
+      </c>
+      <c r="D153" s="10" t="s">
         <v>652</v>
-      </c>
-      <c r="D153" s="10" t="s">
-        <v>653</v>
       </c>
       <c r="E153" s="10" t="s">
         <v>59</v>
@@ -8086,7 +8081,7 @@
         <v>29</v>
       </c>
       <c r="G153" s="10" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="H153" s="10" t="s">
         <v>31</v>
@@ -8095,12 +8090,12 @@
         <v>215</v>
       </c>
       <c r="J153" s="10" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="K153" s="10"/>
       <c r="L153" s="12"/>
       <c r="M153" s="13" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8108,13 +8103,13 @@
         <v>146</v>
       </c>
       <c r="C154" s="10" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D154" s="10" t="s">
+        <v>655</v>
+      </c>
+      <c r="E154" s="10" t="s">
         <v>656</v>
-      </c>
-      <c r="E154" s="10" t="s">
-        <v>657</v>
       </c>
       <c r="F154" s="11" t="s">
         <v>29</v>
@@ -8129,12 +8124,12 @@
         <v>215</v>
       </c>
       <c r="J154" s="10" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="K154" s="10"/>
       <c r="L154" s="12"/>
       <c r="M154" s="13" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8142,33 +8137,33 @@
         <v>147</v>
       </c>
       <c r="C155" s="10" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D155" s="10" t="s">
+        <v>658</v>
+      </c>
+      <c r="E155" s="10" t="s">
         <v>659</v>
       </c>
-      <c r="E155" s="10" t="s">
+      <c r="F155" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G155" s="10" t="s">
+        <v>573</v>
+      </c>
+      <c r="H155" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I155" s="10" t="s">
         <v>660</v>
       </c>
-      <c r="F155" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G155" s="10" t="s">
-        <v>574</v>
-      </c>
-      <c r="H155" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I155" s="10" t="s">
+      <c r="J155" s="10" t="s">
         <v>661</v>
-      </c>
-      <c r="J155" s="10" t="s">
-        <v>662</v>
       </c>
       <c r="K155" s="10"/>
       <c r="L155" s="12"/>
       <c r="M155" s="13" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8176,10 +8171,10 @@
         <v>148</v>
       </c>
       <c r="C156" s="10" t="s">
+        <v>663</v>
+      </c>
+      <c r="D156" s="10" t="s">
         <v>664</v>
-      </c>
-      <c r="D156" s="10" t="s">
-        <v>665</v>
       </c>
       <c r="E156" s="10" t="s">
         <v>59</v>
@@ -8194,17 +8189,17 @@
         <v>206</v>
       </c>
       <c r="I156" s="10" t="s">
+        <v>665</v>
+      </c>
+      <c r="J156" s="10" t="s">
         <v>666</v>
       </c>
-      <c r="J156" s="10" t="s">
+      <c r="K156" s="10" t="s">
         <v>667</v>
-      </c>
-      <c r="K156" s="10" t="s">
-        <v>668</v>
       </c>
       <c r="L156" s="12"/>
       <c r="M156" s="13" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8212,13 +8207,13 @@
         <v>149</v>
       </c>
       <c r="C157" s="10" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="D157" s="10" t="s">
+        <v>669</v>
+      </c>
+      <c r="E157" s="10" t="s">
         <v>670</v>
-      </c>
-      <c r="E157" s="10" t="s">
-        <v>671</v>
       </c>
       <c r="F157" s="11" t="s">
         <v>29</v>
@@ -8230,13 +8225,13 @@
         <v>31</v>
       </c>
       <c r="I157" s="10" t="s">
+        <v>671</v>
+      </c>
+      <c r="J157" s="10" t="s">
         <v>672</v>
       </c>
-      <c r="J157" s="10" t="s">
+      <c r="K157" s="10" t="s">
         <v>673</v>
-      </c>
-      <c r="K157" s="10" t="s">
-        <v>674</v>
       </c>
       <c r="L157" s="12"/>
       <c r="M157" s="13" t="s">
@@ -8248,13 +8243,13 @@
         <v>150</v>
       </c>
       <c r="C158" s="10" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="D158" s="10" t="s">
+        <v>674</v>
+      </c>
+      <c r="E158" s="10" t="s">
         <v>675</v>
-      </c>
-      <c r="E158" s="10" t="s">
-        <v>676</v>
       </c>
       <c r="F158" s="11" t="s">
         <v>29</v>
@@ -8266,10 +8261,10 @@
         <v>31</v>
       </c>
       <c r="I158" s="10" t="s">
+        <v>676</v>
+      </c>
+      <c r="J158" s="10" t="s">
         <v>677</v>
-      </c>
-      <c r="J158" s="10" t="s">
-        <v>678</v>
       </c>
       <c r="K158" s="10"/>
       <c r="L158" s="12"/>
@@ -8327,7 +8322,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="14" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8335,22 +8330,22 @@
         <v>15</v>
       </c>
       <c r="C4" s="16" t="s">
+        <v>679</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>432</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>297</v>
+      </c>
+      <c r="G4" s="16" t="s">
         <v>680</v>
       </c>
-      <c r="D4" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>220</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>298</v>
-      </c>
-      <c r="G4" s="16" t="s">
+      <c r="H4" s="16" t="s">
         <v>681</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>682</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8566,11 +8561,11 @@
       </c>
       <c r="D12" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B12,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E12" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B12,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B12,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -8582,7 +8577,7 @@
       </c>
       <c r="H12" s="19" t="n">
         <f aca="false">IF(C12&gt;0,D12/C12,0)</f>
-        <v>0.857142857142857</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8595,11 +8590,11 @@
       </c>
       <c r="D13" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B13,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E13" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B13,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B13,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -8611,12 +8606,12 @@
       </c>
       <c r="H13" s="19" t="n">
         <f aca="false">IF(C13&gt;0,D13/C13,0)</f>
-        <v>0.857142857142857</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="17" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C14" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B14)</f>
@@ -8645,7 +8640,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="17" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C15" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B15)</f>
@@ -8674,7 +8669,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="17" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C16" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B16)</f>
@@ -8703,7 +8698,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="17" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C17" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B17)</f>
@@ -8732,7 +8727,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="17" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C18" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B18)</f>
@@ -8761,7 +8756,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="17" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C19" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B19)</f>
@@ -8790,7 +8785,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="17" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C20" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B20)</f>
@@ -8819,7 +8814,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="17" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C21" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B21)</f>
@@ -8848,7 +8843,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="17" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C22" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B22)</f>
@@ -8877,7 +8872,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="17" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C23" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B23)</f>
@@ -8906,7 +8901,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="17" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C24" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B24)</f>
@@ -8935,7 +8930,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="17" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C25" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B25)</f>
@@ -8964,7 +8959,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="17" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C26" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B26)</f>
@@ -8993,7 +8988,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="17" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C27" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B27)</f>
@@ -9022,7 +9017,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="17" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C28" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B28)</f>
@@ -9312,7 +9307,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="17" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="C38" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B38)</f>
@@ -9341,7 +9336,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="17" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C39" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B39)</f>
@@ -9370,7 +9365,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="17" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C40" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B40)</f>
@@ -9399,7 +9394,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="17" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="C41" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B41)</f>
@@ -9428,7 +9423,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="17" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="C42" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B42)</f>
@@ -9457,7 +9452,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="17" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C43" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B43)</f>
@@ -9486,7 +9481,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="17" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="C44" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B44)</f>
@@ -9515,7 +9510,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="17" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="C45" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B45)</f>
@@ -9544,7 +9539,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="17" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="C46" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B46)</f>
@@ -9573,7 +9568,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="17" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="C47" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B47)</f>
@@ -9602,7 +9597,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="17" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="C48" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B48)</f>
@@ -9631,7 +9626,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="17" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="C49" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B49)</f>
@@ -9660,7 +9655,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="20" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="C50" s="21" t="n">
         <f aca="false">SUM(C5:C49)</f>
@@ -9668,11 +9663,11 @@
       </c>
       <c r="D50" s="21" t="n">
         <f aca="false">SUM(D5:D49)</f>
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E50" s="21" t="n">
         <f aca="false">SUM(E5:E49)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F50" s="21" t="n">
         <f aca="false">SUM(F5:F49)</f>
@@ -9684,7 +9679,7 @@
       </c>
       <c r="H50" s="22" t="n">
         <f aca="false">IF(C50&gt;0,D50/C50,0)</f>
-        <v>0.946666666666667</v>
+        <v>0.96</v>
       </c>
     </row>
   </sheetData>
@@ -9715,18 +9710,18 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="14" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="23" t="s">
+        <v>683</v>
+      </c>
+      <c r="C4" s="23" t="s">
         <v>684</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="23" t="s">
         <v>685</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>686</v>
       </c>
       <c r="E4" s="23" t="s">
         <v>18</v>
@@ -9734,41 +9729,41 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="24" t="s">
+        <v>686</v>
+      </c>
+      <c r="C5" s="24" t="s">
         <v>687</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="D5" s="24" t="s">
         <v>688</v>
       </c>
-      <c r="D5" s="24" t="s">
-        <v>689</v>
-      </c>
       <c r="E5" s="25" t="s">
-        <v>220</v>
+        <v>432</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="24" t="s">
+        <v>689</v>
+      </c>
+      <c r="C6" s="24" t="s">
         <v>690</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="D6" s="24" t="s">
         <v>691</v>
       </c>
-      <c r="D6" s="24" t="s">
-        <v>692</v>
-      </c>
       <c r="E6" s="25" t="s">
-        <v>220</v>
+        <v>432</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="24" t="s">
+        <v>692</v>
+      </c>
+      <c r="C7" s="24" t="s">
         <v>693</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="D7" s="24" t="s">
         <v>694</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>695</v>
       </c>
       <c r="E7" s="25" t="s">
         <v>29</v>
@@ -9776,41 +9771,41 @@
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="24" t="s">
+        <v>695</v>
+      </c>
+      <c r="C8" s="24" t="s">
         <v>696</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="D8" s="24" t="s">
         <v>697</v>
       </c>
-      <c r="D8" s="24" t="s">
-        <v>698</v>
-      </c>
       <c r="E8" s="25" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="24" t="s">
+        <v>698</v>
+      </c>
+      <c r="C9" s="24" t="s">
         <v>699</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="D9" s="24" t="s">
         <v>700</v>
       </c>
-      <c r="D9" s="24" t="s">
-        <v>701</v>
-      </c>
       <c r="E9" s="25" t="s">
-        <v>220</v>
+        <v>432</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="24" t="s">
+        <v>701</v>
+      </c>
+      <c r="C10" s="24" t="s">
         <v>702</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="D10" s="24" t="s">
         <v>703</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>704</v>
       </c>
       <c r="E10" s="25" t="s">
         <v>29</v>
@@ -9818,44 +9813,44 @@
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="24" t="s">
+        <v>704</v>
+      </c>
+      <c r="C11" s="24" t="s">
         <v>705</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="D11" s="24" t="s">
         <v>706</v>
       </c>
-      <c r="D11" s="24" t="s">
-        <v>707</v>
-      </c>
       <c r="E11" s="25" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="24" t="s">
+        <v>707</v>
+      </c>
+      <c r="C12" s="24" t="s">
         <v>708</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="D12" s="24" t="s">
         <v>709</v>
       </c>
-      <c r="D12" s="24" t="s">
-        <v>710</v>
-      </c>
       <c r="E12" s="25" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="24" t="s">
+        <v>710</v>
+      </c>
+      <c r="C13" s="24" t="s">
         <v>711</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="D13" s="24" t="s">
         <v>712</v>
       </c>
-      <c r="D13" s="24" t="s">
-        <v>713</v>
-      </c>
       <c r="E13" s="25" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -9904,15 +9899,15 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="14" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="26" t="s">
+        <v>714</v>
+      </c>
+      <c r="C4" s="27" t="s">
         <v>715</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>716</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9920,31 +9915,31 @@
         <v>29</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="26" t="s">
-        <v>220</v>
+        <v>432</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="26" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="26" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="52.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9952,7 +9947,7 @@
         <v>21</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9960,15 +9955,15 @@
         <v>22</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="26" t="s">
+        <v>722</v>
+      </c>
+      <c r="C11" s="27" t="s">
         <v>723</v>
-      </c>
-      <c r="C11" s="27" t="s">
-        <v>724</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9976,15 +9971,15 @@
         <v>20</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="26" t="s">
+        <v>725</v>
+      </c>
+      <c r="C13" s="27" t="s">
         <v>726</v>
-      </c>
-      <c r="C13" s="27" t="s">
-        <v>727</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Branded HTML for notification emails; tracker: auto-refill and SMS withdrawal tested on prod
Shopper and brand notification emails use the shared email layout (Open
Nibbl / Open your dashboard buttons); plain-text bodies and subjects
unchanged. Tracker rows #31 and #39 completed after production tests.
</commit_message>
<xml_diff>
--- a/docs/client-requirements/Nibbl_Master_Requirements_Tracker.xlsx
+++ b/docs/client-requirements/Nibbl_Master_Requirements_Tracker.xlsx
@@ -1325,114 +1325,114 @@
     <t xml:space="preserve">Automatic refill (Stripe): trigger 25%, fixed amount, recommendation, failure alert</t>
   </si>
   <si>
+    <t xml:space="preserve">Wallet → Auto-refill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enable auto-refill.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tested on production 13 Oct 2026 in Stripe test mode: $10 top-up with card 4242 credited by webhook; auto-refill enabled in the UI; the auto-refill charge to the saved card credited the wallet; the job skips brands with no recent spend. Live keys are swapped in at go-live (client decision: keep sandbox for testing).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spending Overview + Weekly Statements + detailed ledger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Download a statement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request Refund (Available Cash refundable; reserved/promo not)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand Owner requests up to Available Cash; Nibbl reviews in Admin → Refunds, refunds in Stripe, marks refunded (ledger refund entry) or rejects with a note.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand Dashboard + Admin Dashboard + Backend / API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wallet → Request Refund; Admin → Refunds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request, then mark refunded in Admin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Money is returned manually in Stripe, then recorded here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current plan, recommendation, plan options, scheduled changes, downgrade campaign choice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schedule and cancel a change.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#33, #35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feature comparison table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Side-by-side table (capacity, fees, review cost, identity, CSV, integrations, account manager, early access).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plans → Feature Comparison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open Plans.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan entitlement enforcement (campaign limits, customer identity, CSV, review cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limits, fees, CSV and identity enforced; Starter reviews show first name + last initial and email only on 1–3★.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Covered by tests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#33, #34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Settings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brand Profile (name, website, support email, time zone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Settings → Brand Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change time zone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team &amp; Permissions (Owner / Admin / Viewer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Settings → Team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invite a Viewer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notifications per member (Email + SMS): wallet below 25%, auto-refill failed, campaign paused, exhausted early, new negative review, weekly summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master's six notifications (+ campaign approvals, receipts to review) all sent in-app + email per member preference.</t>
+  </si>
+  <si>
     <t xml:space="preserve">In Progress</t>
   </si>
   <si>
-    <t xml:space="preserve">Wallet → Auto-refill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enable auto-refill.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Production still on Stripe test keys — switch to the live keys received from the client, then retest.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spending Overview + Weekly Statements + detailed ledger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Download a statement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Request Refund (Available Cash refundable; reserved/promo not)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand Owner requests up to Available Cash; Nibbl reviews in Admin → Refunds, refunds in Stripe, marks refunded (ledger refund entry) or rejects with a note.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand Dashboard + Admin Dashboard + Backend / API</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wallet → Request Refund; Admin → Refunds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Request, then mark refunded in Admin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Money is returned manually in Stripe, then recorded here.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current plan, recommendation, plan options, scheduled changes, downgrade campaign choice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Schedule and cancel a change.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#33, #35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feature comparison table</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Side-by-side table (capacity, fees, review cost, identity, CSV, integrations, account manager, early access).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plans → Feature Comparison</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open Plans.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plan entitlement enforcement (campaign limits, customer identity, CSV, review cost)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Limits, fees, CSV and identity enforced; Starter reviews show first name + last initial and email only on 1–3★.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covered by tests.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#33, #34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Settings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brand Profile (name, website, support email, time zone)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Settings → Brand Profile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Change time zone.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Team &amp; Permissions (Owner / Admin / Viewer)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Settings → Team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invite a Viewer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notifications per member (Email + SMS): wallet below 25%, auto-refill failed, campaign paused, exhausted early, new negative review, weekly summary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Master's six notifications (+ campaign approvals, receipts to review) all sent in-app + email per member preference.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Settings → Notifications</t>
   </si>
   <si>
@@ -1631,7 +1631,7 @@
     <t xml:space="preserve">Withdraw a small amount.</t>
   </si>
   <si>
-    <t xml:space="preserve">SMS verification works on production (12 Oct). Do one real website withdrawal with the SMS step, then Completed.</t>
+    <t xml:space="preserve">Tested on production 13 Oct 2026: $1 website withdrawal — amount → locked PayPal → SMS code to a real phone → confirm → Requested (Ready for Batch).</t>
   </si>
   <si>
     <t xml:space="preserve">'Additional review needed' popup; status stays Processing</t>
@@ -2090,10 +2090,10 @@
     <t xml:space="preserve">Our team — Stripe</t>
   </si>
   <si>
-    <t xml:space="preserve">Switch production to the live Stripe keys the client sent; retest checkout, top-up and auto-refill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Client moved Stripe to live production (live keys + webhook secret received)</t>
+    <t xml:space="preserve">Keep Stripe in test mode for testing; swap to the client's live keys at go-live</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top-up and auto-refill tested on production in test mode 13 Oct 2026. Client sandbox keys have no sandbox webhook secret; live keys + live webhook secret received</t>
   </si>
   <si>
     <t xml:space="preserve">Our team — Twilio</t>
@@ -2102,7 +2102,7 @@
     <t xml:space="preserve">Retest SMS-verified withdrawals; lock verified phones (change via admin + history)</t>
   </si>
   <si>
-    <t xml:space="preserve">Twilio SMS verified on production 12 Oct 2026 (code sent to a Bangladesh number, delivered, approved). Remaining: one real website withdrawal with the SMS step</t>
+    <t xml:space="preserve">Twilio SMS verified on production 12 Oct 2026; real website withdrawal with the SMS step completed 13 Oct 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Client — DNS</t>
@@ -3050,11 +3050,11 @@
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"Completed")</f>
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"In Progress")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">COUNTIF(F9:F158,"In Review")</f>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="H5" s="5" t="n">
         <f aca="false">IF(C5&gt;0,D5/C5,0)</f>
-        <v>0.96</v>
+        <v>0.973333333333333</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6408,7 +6408,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B105" s="9" t="n">
         <v>97</v>
       </c>
@@ -6422,7 +6422,7 @@
         <v>59</v>
       </c>
       <c r="F105" s="11" t="s">
-        <v>432</v>
+        <v>29</v>
       </c>
       <c r="G105" s="10" t="s">
         <v>51</v>
@@ -6431,17 +6431,17 @@
         <v>31</v>
       </c>
       <c r="I105" s="10" t="s">
+        <v>432</v>
+      </c>
+      <c r="J105" s="10" t="s">
         <v>433</v>
       </c>
-      <c r="J105" s="10" t="s">
+      <c r="K105" s="10" t="s">
         <v>434</v>
-      </c>
-      <c r="K105" s="10" t="s">
-        <v>435</v>
       </c>
       <c r="L105" s="12"/>
       <c r="M105" s="13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6452,7 +6452,7 @@
         <v>423</v>
       </c>
       <c r="D106" s="10" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="E106" s="10" t="s">
         <v>59</v>
@@ -6470,12 +6470,12 @@
         <v>425</v>
       </c>
       <c r="J106" s="10" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="K106" s="10"/>
       <c r="L106" s="12"/>
       <c r="M106" s="13" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6486,28 +6486,28 @@
         <v>423</v>
       </c>
       <c r="D107" s="10" t="s">
+        <v>439</v>
+      </c>
+      <c r="E107" s="10" t="s">
         <v>440</v>
       </c>
-      <c r="E107" s="10" t="s">
+      <c r="F107" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G107" s="10" t="s">
         <v>441</v>
       </c>
-      <c r="F107" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G107" s="10" t="s">
+      <c r="H107" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I107" s="10" t="s">
         <v>442</v>
       </c>
-      <c r="H107" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I107" s="10" t="s">
+      <c r="J107" s="10" t="s">
         <v>443</v>
       </c>
-      <c r="J107" s="10" t="s">
+      <c r="K107" s="10" t="s">
         <v>444</v>
-      </c>
-      <c r="K107" s="10" t="s">
-        <v>445</v>
       </c>
       <c r="L107" s="12"/>
       <c r="M107" s="13" t="s">
@@ -6519,10 +6519,10 @@
         <v>100</v>
       </c>
       <c r="C108" s="10" t="s">
+        <v>445</v>
+      </c>
+      <c r="D108" s="10" t="s">
         <v>446</v>
-      </c>
-      <c r="D108" s="10" t="s">
-        <v>447</v>
       </c>
       <c r="E108" s="10" t="s">
         <v>59</v>
@@ -6537,15 +6537,15 @@
         <v>31</v>
       </c>
       <c r="I108" s="10" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="J108" s="10" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="K108" s="10"/>
       <c r="L108" s="12"/>
       <c r="M108" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6553,13 +6553,13 @@
         <v>101</v>
       </c>
       <c r="C109" s="10" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="D109" s="10" t="s">
+        <v>449</v>
+      </c>
+      <c r="E109" s="10" t="s">
         <v>450</v>
-      </c>
-      <c r="E109" s="10" t="s">
-        <v>451</v>
       </c>
       <c r="F109" s="11" t="s">
         <v>29</v>
@@ -6571,10 +6571,10 @@
         <v>31</v>
       </c>
       <c r="I109" s="10" t="s">
+        <v>451</v>
+      </c>
+      <c r="J109" s="10" t="s">
         <v>452</v>
-      </c>
-      <c r="J109" s="10" t="s">
-        <v>453</v>
       </c>
       <c r="K109" s="10"/>
       <c r="L109" s="12"/>
@@ -6587,13 +6587,13 @@
         <v>102</v>
       </c>
       <c r="C110" s="10" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="D110" s="10" t="s">
+        <v>453</v>
+      </c>
+      <c r="E110" s="10" t="s">
         <v>454</v>
-      </c>
-      <c r="E110" s="10" t="s">
-        <v>455</v>
       </c>
       <c r="F110" s="11" t="s">
         <v>29</v>
@@ -6608,12 +6608,12 @@
         <v>172</v>
       </c>
       <c r="J110" s="10" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="K110" s="10"/>
       <c r="L110" s="12"/>
       <c r="M110" s="13" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6621,10 +6621,10 @@
         <v>103</v>
       </c>
       <c r="C111" s="10" t="s">
+        <v>457</v>
+      </c>
+      <c r="D111" s="10" t="s">
         <v>458</v>
-      </c>
-      <c r="D111" s="10" t="s">
-        <v>459</v>
       </c>
       <c r="E111" s="10" t="s">
         <v>59</v>
@@ -6639,15 +6639,15 @@
         <v>31</v>
       </c>
       <c r="I111" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="J111" s="10" t="s">
         <v>460</v>
-      </c>
-      <c r="J111" s="10" t="s">
-        <v>461</v>
       </c>
       <c r="K111" s="10"/>
       <c r="L111" s="12"/>
       <c r="M111" s="13" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6655,10 +6655,10 @@
         <v>104</v>
       </c>
       <c r="C112" s="10" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D112" s="10" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="E112" s="10" t="s">
         <v>59</v>
@@ -6673,15 +6673,15 @@
         <v>31</v>
       </c>
       <c r="I112" s="10" t="s">
+        <v>463</v>
+      </c>
+      <c r="J112" s="10" t="s">
         <v>464</v>
-      </c>
-      <c r="J112" s="10" t="s">
-        <v>465</v>
       </c>
       <c r="K112" s="10"/>
       <c r="L112" s="12"/>
       <c r="M112" s="13" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6689,16 +6689,16 @@
         <v>105</v>
       </c>
       <c r="C113" s="10" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D113" s="10" t="s">
+        <v>465</v>
+      </c>
+      <c r="E113" s="10" t="s">
         <v>466</v>
       </c>
-      <c r="E113" s="10" t="s">
+      <c r="F113" s="11" t="s">
         <v>467</v>
-      </c>
-      <c r="F113" s="11" t="s">
-        <v>432</v>
       </c>
       <c r="G113" s="10" t="s">
         <v>51</v>
@@ -6717,7 +6717,7 @@
       </c>
       <c r="L113" s="12"/>
       <c r="M113" s="13" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6725,7 +6725,7 @@
         <v>106</v>
       </c>
       <c r="C114" s="10" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D114" s="10" t="s">
         <v>471</v>
@@ -6759,7 +6759,7 @@
         <v>107</v>
       </c>
       <c r="C115" s="10" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D115" s="10" t="s">
         <v>474</v>
@@ -6785,7 +6785,7 @@
       <c r="K115" s="10"/>
       <c r="L115" s="12"/>
       <c r="M115" s="13" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6793,7 +6793,7 @@
         <v>108</v>
       </c>
       <c r="C116" s="10" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D116" s="10" t="s">
         <v>478</v>
@@ -6819,7 +6819,7 @@
       <c r="K116" s="10"/>
       <c r="L116" s="12"/>
       <c r="M116" s="13" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7248,7 +7248,7 @@
         <v>531</v>
       </c>
       <c r="F129" s="11" t="s">
-        <v>432</v>
+        <v>29</v>
       </c>
       <c r="G129" s="10" t="s">
         <v>205</v>
@@ -7398,7 +7398,7 @@
         <v>553</v>
       </c>
       <c r="J133" s="10" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="K133" s="10"/>
       <c r="L133" s="12"/>
@@ -8336,7 +8336,7 @@
         <v>29</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>432</v>
+        <v>467</v>
       </c>
       <c r="F4" s="16" t="s">
         <v>297</v>
@@ -9025,11 +9025,11 @@
       </c>
       <c r="D28" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B28,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E28" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B28,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B28,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -9041,12 +9041,12 @@
       </c>
       <c r="H28" s="19" t="n">
         <f aca="false">IF(C28&gt;0,D28/C28,0)</f>
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="17" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C29" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B29)</f>
@@ -9075,7 +9075,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="17" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C30" s="18" t="n">
         <f aca="false">COUNTIF('Master Requirements Tracker'!$C$9:$C$158,B30)</f>
@@ -9199,11 +9199,11 @@
       </c>
       <c r="D34" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B34,'Master Requirements Tracker'!$F$9:$F$158,"Completed")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E34" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B34,'Master Requirements Tracker'!$F$9:$F$158,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34" s="18" t="n">
         <f aca="false">COUNTIFS('Master Requirements Tracker'!$C$9:$C$158,B34,'Master Requirements Tracker'!$F$9:$F$158,"In Review")</f>
@@ -9215,7 +9215,7 @@
       </c>
       <c r="H34" s="19" t="n">
         <f aca="false">IF(C34&gt;0,D34/C34,0)</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9663,11 +9663,11 @@
       </c>
       <c r="D50" s="21" t="n">
         <f aca="false">SUM(D5:D49)</f>
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E50" s="21" t="n">
         <f aca="false">SUM(E5:E49)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F50" s="21" t="n">
         <f aca="false">SUM(F5:F49)</f>
@@ -9679,7 +9679,7 @@
       </c>
       <c r="H50" s="22" t="n">
         <f aca="false">IF(C50&gt;0,D50/C50,0)</f>
-        <v>0.96</v>
+        <v>0.973333333333333</v>
       </c>
     </row>
   </sheetData>
@@ -9738,7 +9738,7 @@
         <v>688</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>432</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9752,7 +9752,7 @@
         <v>691</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>432</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9794,7 +9794,7 @@
         <v>700</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>432</v>
+        <v>467</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9920,7 +9920,7 @@
     </row>
     <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="26" t="s">
-        <v>432</v>
+        <v>467</v>
       </c>
       <c r="C6" s="27" t="s">
         <v>717</v>

</xml_diff>